<commit_message>
Catálogo: agregar 30 productos más de CW & BW
- Sartenes, juegos, ollas/cazos y baterías nuevas (69 productos en total).
- Nueva categoría 'Ollas y cazos'.
- Imágenes PNG divididas por grupo de categorías para que se lean bien
  en el celular (sartenes / ollas y baterías / licuadoras y más).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FUhhJ2BRdUSntnn7uyZg21
</commit_message>
<xml_diff>
--- a/catalogo-cocina/salida/precios_internos_cocina.xlsx
+++ b/catalogo-cocina/salida/precios_internos_cocina.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Pendientes" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Precios!$A$4:$N$43</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Precios!$A$4:$N$73</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +31,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="F44" authorId="0">
+    <comment ref="F74" authorId="0">
       <text>
         <r>
           <rPr>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="199">
   <si>
     <t xml:space="preserve">Lista de precios interna (NO compartir con clientes)</t>
   </si>
@@ -110,24 +110,48 @@
     <t xml:space="preserve">Sartén Character Roja 20 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP20 J GT HEALTHY COOK GREY HIPPO MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Healthy Cook Gris 20 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">SARTEN 20 CM RJ VITAL FR</t>
   </si>
   <si>
     <t xml:space="preserve">Sartén Vital Roja 20 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP24 J LY ESSENTIAL TITA VIOLINE GR MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Essential Titanium Gris 24 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">SARTEN 28 CM RJ CHARACTER</t>
   </si>
   <si>
     <t xml:space="preserve">Sartén Character Roja 28 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP26 J LY ESSENTIAL TITA VIOLINE GR MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Essential Titanium Gris 26 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">SARTEN 24 CM RJ VITAL FR</t>
   </si>
   <si>
     <t xml:space="preserve">Sartén Vital Roja 24 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP26 J LYON SIMPLICITY BLACK T-FAL MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Simplicity Negra 26 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">SARTEN 26 CM RJ VITAL FR</t>
   </si>
   <si>
@@ -140,42 +164,186 @@
     <t xml:space="preserve">Sartén Trendy Titanium 20 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP20 B UNI PE G6 DELIGHT IND BEIGE SAND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Delight Beige 20 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">SARTEN 24 CM TRENDY TITANIUM</t>
   </si>
   <si>
     <t xml:space="preserve">Sartén Trendy Titanium 24 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP26 GOUR NOM INTUITION G6 SS POLI GB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Intuition 26 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">CREPERA 25 CM HARD TIT EXPERT</t>
   </si>
   <si>
     <t xml:space="preserve">Crepera Hard Titanium Expert 25 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP24 B SOFIA PE G6 DELIGHT IND BEIGE SAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Delight Beige 24 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FP28 B SOFIA PE G6 DELIGHT IND BEIGE SAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Delight Beige 28 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FP30 GOUR NOM INTUITION G6 SS COAT MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Intuition 30 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Juegos de sartenes</t>
   </si>
   <si>
+    <t xml:space="preserve">JGO STN 20/24 CM NGO EASY CARE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 2 sartenes Easy Care Negro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET FP20/24 G6 E-CARE RED SURP T-F MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 2 sartenes Easy Care Rojo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET SRTNS 20/28CM NG FR 2022 EASY CARE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET FP20+PCKP25 HEALTHY COOK GR HIPPO MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set Healthy Cook Gris: sartén + crepera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JGO 24/30 RJ SIMPLY TITANIUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 2 sartenes Simply Titanium Rojo</t>
+  </si>
+  <si>
     <t xml:space="preserve">JGO 20/24/28 CM ROJO CHARACTER</t>
   </si>
   <si>
     <t xml:space="preserve">Juego de 3 sartenes Character Rojo</t>
   </si>
   <si>
+    <t xml:space="preserve">JGO 20/24/30 RJ SIMPLY TITANIUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 3 sartenes Simply Titanium Rojo</t>
+  </si>
+  <si>
     <t xml:space="preserve">JGO 12/20/24/26 CM RJO VITAL</t>
   </si>
   <si>
     <t xml:space="preserve">Juego de 4 sartenes Vital Rojo</t>
   </si>
   <si>
+    <t xml:space="preserve">SET 3P HANAE HARD TITANIUM + BLACK MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 3 sartenes Hard Titanium+ Black</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET 20/28 CM VIN RESIST INTENSE CLUBS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 2 sartenes Resist Intense</t>
+  </si>
+  <si>
     <t xml:space="preserve">JGO 20/24/28 CM BG TRENDY TITANIUM</t>
   </si>
   <si>
     <t xml:space="preserve">Juego de 3 sartenes Trendy Titanium Beige</t>
   </si>
   <si>
+    <t xml:space="preserve">JGO STN 20/24/28 CM DAILY EXPERT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 3 sartenes Daily Expert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ollas y cazos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAZO 16 CM C/T ROJO SIMPLY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cazo Simply Rojo 16 cm con tapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MILK POT14 B STR HARD TITANIUM +BLACK MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lechera Hard Titanium+ Black 14 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAZO 18 CM C/T EASY TITANIUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cazo Easy Titanium 18 cm con tapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCP20LID B LENA HARD TITANIUM + BLACK MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cazo Hard Titanium+ Black 20 cm con tapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D.OV24LID LENEXLOW COCINA LIMP DRESS BLU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Olla Azul 24 cm con tapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STW24LID B LENA HARD TITANIUM + BLACK MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Olla Hard Titanium+ Black 24 cm con tapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OLLA 20 CM C/T TRENDY TITANIUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Olla Trendy Titanium 20 cm con tapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OLLA 24 CM C/T C/C DELIGHT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Olla Delight Beige 24 cm con tapa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Baterías de cocina</t>
   </si>
   <si>
+    <t xml:space="preserve">BAT 5 PZS NEGRA EASY CARE VIET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batería Easy Care Negra 5 piezas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAT 11 PZS EXPERT CHEF BF MAYOREO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batería Expert Chef 11 piezas</t>
+  </si>
+  <si>
     <t xml:space="preserve">BAT 9 PZS LIC NEGRA SUPERCOOK V2</t>
   </si>
   <si>
@@ -198,6 +366,18 @@
   </si>
   <si>
     <t xml:space="preserve">Batería Excite Azul 14 piezas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BATERIA INOX 6 PCS INTUITION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batería Intuition 6 piezas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BATERIA 12PZS NERA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batería Negra 12 piezas</t>
   </si>
   <si>
     <t xml:space="preserve">Food Prep</t>
@@ -1042,7 +1222,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N74"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1192,7 +1372,7 @@
         <v>21</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>126.08</v>
+        <v>109.36</v>
       </c>
       <c r="G6" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F6,Reglas!$A$5:$A$8,1))</f>
@@ -1205,23 +1385,23 @@
       </c>
       <c r="J6" s="9" t="n">
         <f aca="false">IF(H6="",MAX(F6*(1+G6),I6),F6*(1+H6))</f>
-        <v>226.944</v>
+        <v>196.848</v>
       </c>
       <c r="K6" s="10" t="n">
         <f aca="false">IF(J6&lt;1000,CEILING(J6,10)-1,CEILING(J6,50)-1)</f>
-        <v>229</v>
+        <v>199</v>
       </c>
       <c r="L6" s="9" t="n">
         <f aca="false">K6-F6</f>
-        <v>102.92</v>
+        <v>89.64</v>
       </c>
       <c r="M6" s="11" t="n">
         <f aca="false">IF(K6=0,"",L6/K6)</f>
-        <v>0.44943231441048</v>
+        <v>0.450452261306533</v>
       </c>
       <c r="N6" s="11" t="n">
         <f aca="false">IF(F6=0,"",K6/F6-1)</f>
-        <v>0.816307106598985</v>
+        <v>0.819678127286028</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1241,7 +1421,7 @@
         <v>23</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>141.55</v>
+        <v>126.08</v>
       </c>
       <c r="G7" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F7,Reglas!$A$5:$A$8,1))</f>
@@ -1254,23 +1434,23 @@
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">IF(H7="",MAX(F7*(1+G7),I7),F7*(1+H7))</f>
-        <v>254.79</v>
+        <v>226.944</v>
       </c>
       <c r="K7" s="10" t="n">
         <f aca="false">IF(J7&lt;1000,CEILING(J7,10)-1,CEILING(J7,50)-1)</f>
-        <v>259</v>
+        <v>229</v>
       </c>
       <c r="L7" s="9" t="n">
         <f aca="false">K7-F7</f>
-        <v>117.45</v>
+        <v>102.92</v>
       </c>
       <c r="M7" s="11" t="n">
         <f aca="false">IF(K7=0,"",L7/K7)</f>
-        <v>0.453474903474903</v>
+        <v>0.44943231441048</v>
       </c>
       <c r="N7" s="11" t="n">
         <f aca="false">IF(F7=0,"",K7/F7-1)</f>
-        <v>0.829742140586365</v>
+        <v>0.816307106598985</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1290,7 +1470,7 @@
         <v>25</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>146.67</v>
+        <v>128.23</v>
       </c>
       <c r="G8" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F8,Reglas!$A$5:$A$8,1))</f>
@@ -1303,23 +1483,23 @@
       </c>
       <c r="J8" s="9" t="n">
         <f aca="false">IF(H8="",MAX(F8*(1+G8),I8),F8*(1+H8))</f>
-        <v>264.006</v>
+        <v>230.814</v>
       </c>
       <c r="K8" s="10" t="n">
         <f aca="false">IF(J8&lt;1000,CEILING(J8,10)-1,CEILING(J8,50)-1)</f>
-        <v>269</v>
+        <v>239</v>
       </c>
       <c r="L8" s="9" t="n">
         <f aca="false">K8-F8</f>
-        <v>122.33</v>
+        <v>110.77</v>
       </c>
       <c r="M8" s="11" t="n">
         <f aca="false">IF(K8=0,"",L8/K8)</f>
-        <v>0.454758364312268</v>
+        <v>0.46347280334728</v>
       </c>
       <c r="N8" s="11" t="n">
         <f aca="false">IF(F8=0,"",K8/F8-1)</f>
-        <v>0.834049226153951</v>
+        <v>0.863838415347423</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1339,7 +1519,7 @@
         <v>27</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>158.83</v>
+        <v>141.55</v>
       </c>
       <c r="G9" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F9,Reglas!$A$5:$A$8,1))</f>
@@ -1352,23 +1532,23 @@
       </c>
       <c r="J9" s="9" t="n">
         <f aca="false">IF(H9="",MAX(F9*(1+G9),I9),F9*(1+H9))</f>
-        <v>285.894</v>
+        <v>254.79</v>
       </c>
       <c r="K9" s="10" t="n">
         <f aca="false">IF(J9&lt;1000,CEILING(J9,10)-1,CEILING(J9,50)-1)</f>
-        <v>289</v>
+        <v>259</v>
       </c>
       <c r="L9" s="9" t="n">
         <f aca="false">K9-F9</f>
-        <v>130.17</v>
+        <v>117.45</v>
       </c>
       <c r="M9" s="11" t="n">
         <f aca="false">IF(K9=0,"",L9/K9)</f>
-        <v>0.450415224913495</v>
+        <v>0.453474903474903</v>
       </c>
       <c r="N9" s="11" t="n">
         <f aca="false">IF(F9=0,"",K9/F9-1)</f>
-        <v>0.819555499590757</v>
+        <v>0.829742140586365</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1388,7 +1568,7 @@
         <v>29</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>202.07</v>
+        <v>140.1</v>
       </c>
       <c r="G10" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F10,Reglas!$A$5:$A$8,1))</f>
@@ -1401,23 +1581,23 @@
       </c>
       <c r="J10" s="9" t="n">
         <f aca="false">IF(H10="",MAX(F10*(1+G10),I10),F10*(1+H10))</f>
-        <v>363.726</v>
+        <v>252.18</v>
       </c>
       <c r="K10" s="10" t="n">
         <f aca="false">IF(J10&lt;1000,CEILING(J10,10)-1,CEILING(J10,50)-1)</f>
-        <v>369</v>
+        <v>259</v>
       </c>
       <c r="L10" s="9" t="n">
         <f aca="false">K10-F10</f>
-        <v>166.93</v>
+        <v>118.9</v>
       </c>
       <c r="M10" s="11" t="n">
         <f aca="false">IF(K10=0,"",L10/K10)</f>
-        <v>0.452384823848239</v>
+        <v>0.459073359073359</v>
       </c>
       <c r="N10" s="11" t="n">
         <f aca="false">IF(F10=0,"",K10/F10-1)</f>
-        <v>0.826099866382937</v>
+        <v>0.848679514632406</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1437,7 +1617,7 @@
         <v>31</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>216.46</v>
+        <v>146.67</v>
       </c>
       <c r="G11" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F11,Reglas!$A$5:$A$8,1))</f>
@@ -1450,23 +1630,23 @@
       </c>
       <c r="J11" s="9" t="n">
         <f aca="false">IF(H11="",MAX(F11*(1+G11),I11),F11*(1+H11))</f>
-        <v>389.628</v>
+        <v>264.006</v>
       </c>
       <c r="K11" s="10" t="n">
         <f aca="false">IF(J11&lt;1000,CEILING(J11,10)-1,CEILING(J11,50)-1)</f>
-        <v>389</v>
+        <v>269</v>
       </c>
       <c r="L11" s="9" t="n">
         <f aca="false">K11-F11</f>
-        <v>172.54</v>
+        <v>122.33</v>
       </c>
       <c r="M11" s="11" t="n">
         <f aca="false">IF(K11=0,"",L11/K11)</f>
-        <v>0.443547557840617</v>
+        <v>0.454758364312268</v>
       </c>
       <c r="N11" s="11" t="n">
         <f aca="false">IF(F11=0,"",K11/F11-1)</f>
-        <v>0.797098771135545</v>
+        <v>0.834049226153951</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1486,7 +1666,7 @@
         <v>33</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>229.98</v>
+        <v>151.2</v>
       </c>
       <c r="G12" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F12,Reglas!$A$5:$A$8,1))</f>
@@ -1499,23 +1679,23 @@
       </c>
       <c r="J12" s="9" t="n">
         <f aca="false">IF(H12="",MAX(F12*(1+G12),I12),F12*(1+H12))</f>
-        <v>413.964</v>
+        <v>272.16</v>
       </c>
       <c r="K12" s="10" t="n">
         <f aca="false">IF(J12&lt;1000,CEILING(J12,10)-1,CEILING(J12,50)-1)</f>
-        <v>419</v>
+        <v>279</v>
       </c>
       <c r="L12" s="9" t="n">
         <f aca="false">K12-F12</f>
-        <v>189.02</v>
+        <v>127.8</v>
       </c>
       <c r="M12" s="11" t="n">
         <f aca="false">IF(K12=0,"",L12/K12)</f>
-        <v>0.451121718377088</v>
+        <v>0.458064516129032</v>
       </c>
       <c r="N12" s="11" t="n">
         <f aca="false">IF(F12=0,"",K12/F12-1)</f>
-        <v>0.821897556309244</v>
+        <v>0.845238095238095</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1526,45 +1706,45 @@
         <v>16</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="F13" s="5" t="n">
-        <v>362.45</v>
+        <v>158.83</v>
       </c>
       <c r="G13" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F13,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H13" s="7"/>
       <c r="I13" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F13,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J13" s="9" t="n">
         <f aca="false">IF(H13="",MAX(F13*(1+G13),I13),F13*(1+H13))</f>
-        <v>598.0425</v>
+        <v>285.894</v>
       </c>
       <c r="K13" s="10" t="n">
         <f aca="false">IF(J13&lt;1000,CEILING(J13,10)-1,CEILING(J13,50)-1)</f>
-        <v>599</v>
+        <v>289</v>
       </c>
       <c r="L13" s="9" t="n">
         <f aca="false">K13-F13</f>
-        <v>236.55</v>
+        <v>130.17</v>
       </c>
       <c r="M13" s="11" t="n">
         <f aca="false">IF(K13=0,"",L13/K13)</f>
-        <v>0.394908180300501</v>
+        <v>0.450415224913495</v>
       </c>
       <c r="N13" s="11" t="n">
         <f aca="false">IF(F13=0,"",K13/F13-1)</f>
-        <v>0.652641743688785</v>
+        <v>0.819555499590757</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1575,45 +1755,45 @@
         <v>16</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="F14" s="5" t="n">
-        <v>492.72</v>
+        <v>202.07</v>
       </c>
       <c r="G14" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F14,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H14" s="7"/>
       <c r="I14" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F14,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J14" s="9" t="n">
         <f aca="false">IF(H14="",MAX(F14*(1+G14),I14),F14*(1+H14))</f>
-        <v>812.988</v>
+        <v>363.726</v>
       </c>
       <c r="K14" s="10" t="n">
         <f aca="false">IF(J14&lt;1000,CEILING(J14,10)-1,CEILING(J14,50)-1)</f>
-        <v>819</v>
+        <v>369</v>
       </c>
       <c r="L14" s="9" t="n">
         <f aca="false">K14-F14</f>
-        <v>326.28</v>
+        <v>166.93</v>
       </c>
       <c r="M14" s="11" t="n">
         <f aca="false">IF(K14=0,"",L14/K14)</f>
-        <v>0.398388278388278</v>
+        <v>0.452384823848239</v>
       </c>
       <c r="N14" s="11" t="n">
         <f aca="false">IF(F14=0,"",K14/F14-1)</f>
-        <v>0.662201656113005</v>
+        <v>0.826099866382937</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1624,45 +1804,45 @@
         <v>16</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D15" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="F15" s="5" t="n">
-        <v>705.08</v>
+        <v>214.17</v>
       </c>
       <c r="G15" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F15,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.8</v>
       </c>
       <c r="H15" s="7"/>
       <c r="I15" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F15,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>0</v>
       </c>
       <c r="J15" s="9" t="n">
         <f aca="false">IF(H15="",MAX(F15*(1+G15),I15),F15*(1+H15))</f>
-        <v>1155</v>
+        <v>385.506</v>
       </c>
       <c r="K15" s="10" t="n">
         <f aca="false">IF(J15&lt;1000,CEILING(J15,10)-1,CEILING(J15,50)-1)</f>
-        <v>1199</v>
+        <v>389</v>
       </c>
       <c r="L15" s="9" t="n">
         <f aca="false">K15-F15</f>
-        <v>493.92</v>
+        <v>174.83</v>
       </c>
       <c r="M15" s="11" t="n">
         <f aca="false">IF(K15=0,"",L15/K15)</f>
-        <v>0.411943286071726</v>
+        <v>0.449434447300771</v>
       </c>
       <c r="N15" s="11" t="n">
         <f aca="false">IF(F15=0,"",K15/F15-1)</f>
-        <v>0.700516253474783</v>
+        <v>0.816314142970538</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,45 +1853,45 @@
         <v>16</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="F16" s="5" t="n">
-        <v>866.93</v>
+        <v>216.46</v>
       </c>
       <c r="G16" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F16,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.8</v>
       </c>
       <c r="H16" s="7"/>
       <c r="I16" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F16,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>0</v>
       </c>
       <c r="J16" s="9" t="n">
         <f aca="false">IF(H16="",MAX(F16*(1+G16),I16),F16*(1+H16))</f>
-        <v>1343.7415</v>
+        <v>389.628</v>
       </c>
       <c r="K16" s="10" t="n">
         <f aca="false">IF(J16&lt;1000,CEILING(J16,10)-1,CEILING(J16,50)-1)</f>
-        <v>1349</v>
+        <v>389</v>
       </c>
       <c r="L16" s="9" t="n">
         <f aca="false">K16-F16</f>
-        <v>482.07</v>
+        <v>172.54</v>
       </c>
       <c r="M16" s="11" t="n">
         <f aca="false">IF(K16=0,"",L16/K16)</f>
-        <v>0.357353595255745</v>
+        <v>0.443547557840617</v>
       </c>
       <c r="N16" s="11" t="n">
         <f aca="false">IF(F16=0,"",K16/F16-1)</f>
-        <v>0.556065656973458</v>
+        <v>0.797098771135545</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1722,45 +1902,45 @@
         <v>16</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>901.39</v>
+        <v>226.69</v>
       </c>
       <c r="G17" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F17,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.8</v>
       </c>
       <c r="H17" s="7"/>
       <c r="I17" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F17,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>0</v>
       </c>
       <c r="J17" s="9" t="n">
         <f aca="false">IF(H17="",MAX(F17*(1+G17),I17),F17*(1+H17))</f>
-        <v>1397.1545</v>
+        <v>408.042</v>
       </c>
       <c r="K17" s="10" t="n">
         <f aca="false">IF(J17&lt;1000,CEILING(J17,10)-1,CEILING(J17,50)-1)</f>
-        <v>1399</v>
+        <v>409</v>
       </c>
       <c r="L17" s="9" t="n">
         <f aca="false">K17-F17</f>
-        <v>497.61</v>
+        <v>182.31</v>
       </c>
       <c r="M17" s="11" t="n">
         <f aca="false">IF(K17=0,"",L17/K17)</f>
-        <v>0.355689778413152</v>
+        <v>0.445745721271394</v>
       </c>
       <c r="N17" s="11" t="n">
         <f aca="false">IF(F17=0,"",K17/F17-1)</f>
-        <v>0.552047393470085</v>
+        <v>0.804226035555163</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1771,45 +1951,45 @@
         <v>16</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>1012.41</v>
+        <v>229.98</v>
       </c>
       <c r="G18" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F18,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.8</v>
       </c>
       <c r="H18" s="7"/>
       <c r="I18" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F18,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>0</v>
       </c>
       <c r="J18" s="9" t="n">
         <f aca="false">IF(H18="",MAX(F18*(1+G18),I18),F18*(1+H18))</f>
-        <v>1569.2355</v>
+        <v>413.964</v>
       </c>
       <c r="K18" s="10" t="n">
         <f aca="false">IF(J18&lt;1000,CEILING(J18,10)-1,CEILING(J18,50)-1)</f>
-        <v>1599</v>
+        <v>419</v>
       </c>
       <c r="L18" s="9" t="n">
         <f aca="false">K18-F18</f>
-        <v>586.59</v>
+        <v>189.02</v>
       </c>
       <c r="M18" s="11" t="n">
         <f aca="false">IF(K18=0,"",L18/K18)</f>
-        <v>0.366848030018762</v>
+        <v>0.451121718377088</v>
       </c>
       <c r="N18" s="11" t="n">
         <f aca="false">IF(F18=0,"",K18/F18-1)</f>
-        <v>0.57939965033929</v>
+        <v>0.821897556309244</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1820,45 +2000,45 @@
         <v>16</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1047.3</v>
+        <v>254.22</v>
       </c>
       <c r="G19" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F19,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.8</v>
       </c>
       <c r="H19" s="7"/>
       <c r="I19" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F19,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>0</v>
       </c>
       <c r="J19" s="9" t="n">
         <f aca="false">IF(H19="",MAX(F19*(1+G19),I19),F19*(1+H19))</f>
-        <v>1623.315</v>
+        <v>457.596</v>
       </c>
       <c r="K19" s="10" t="n">
         <f aca="false">IF(J19&lt;1000,CEILING(J19,10)-1,CEILING(J19,50)-1)</f>
-        <v>1649</v>
+        <v>459</v>
       </c>
       <c r="L19" s="9" t="n">
         <f aca="false">K19-F19</f>
-        <v>601.7</v>
+        <v>204.78</v>
       </c>
       <c r="M19" s="11" t="n">
         <f aca="false">IF(K19=0,"",L19/K19)</f>
-        <v>0.364887810794421</v>
+        <v>0.446143790849673</v>
       </c>
       <c r="N19" s="11" t="n">
         <f aca="false">IF(F19=0,"",K19/F19-1)</f>
-        <v>0.574524968967822</v>
+        <v>0.805522775548737</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1866,48 +2046,48 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>362.5</v>
+        <v>294.26</v>
       </c>
       <c r="G20" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F20,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H20" s="7"/>
       <c r="I20" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F20,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J20" s="9" t="n">
         <f aca="false">IF(H20="",MAX(F20*(1+G20),I20),F20*(1+H20))</f>
-        <v>598.125</v>
+        <v>529.668</v>
       </c>
       <c r="K20" s="10" t="n">
         <f aca="false">IF(J20&lt;1000,CEILING(J20,10)-1,CEILING(J20,50)-1)</f>
-        <v>599</v>
+        <v>529</v>
       </c>
       <c r="L20" s="9" t="n">
         <f aca="false">K20-F20</f>
-        <v>236.5</v>
+        <v>234.74</v>
       </c>
       <c r="M20" s="11" t="n">
         <f aca="false">IF(K20=0,"",L20/K20)</f>
-        <v>0.394824707846411</v>
+        <v>0.443742911153119</v>
       </c>
       <c r="N20" s="11" t="n">
         <f aca="false">IF(F20=0,"",K20/F20-1)</f>
-        <v>0.652413793103448</v>
+        <v>0.797729898729015</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1915,48 +2095,48 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="E21" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>55</v>
-      </c>
       <c r="F21" s="5" t="n">
-        <v>384.06</v>
+        <v>292.49</v>
       </c>
       <c r="G21" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F21,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H21" s="7"/>
       <c r="I21" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F21,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J21" s="9" t="n">
         <f aca="false">IF(H21="",MAX(F21*(1+G21),I21),F21*(1+H21))</f>
-        <v>633.699</v>
+        <v>526.482</v>
       </c>
       <c r="K21" s="10" t="n">
         <f aca="false">IF(J21&lt;1000,CEILING(J21,10)-1,CEILING(J21,50)-1)</f>
-        <v>639</v>
+        <v>529</v>
       </c>
       <c r="L21" s="9" t="n">
         <f aca="false">K21-F21</f>
-        <v>254.94</v>
+        <v>236.51</v>
       </c>
       <c r="M21" s="11" t="n">
         <f aca="false">IF(K21=0,"",L21/K21)</f>
-        <v>0.398967136150235</v>
+        <v>0.447088846880907</v>
       </c>
       <c r="N21" s="11" t="n">
         <f aca="false">IF(F21=0,"",K21/F21-1)</f>
-        <v>0.663802530854554</v>
+        <v>0.808608841327909</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1964,48 +2144,48 @@
         <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>384.59</v>
+        <v>184</v>
       </c>
       <c r="G22" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F22,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H22" s="7"/>
       <c r="I22" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F22,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J22" s="9" t="n">
         <f aca="false">IF(H22="",MAX(F22*(1+G22),I22),F22*(1+H22))</f>
-        <v>634.5735</v>
+        <v>331.2</v>
       </c>
       <c r="K22" s="10" t="n">
         <f aca="false">IF(J22&lt;1000,CEILING(J22,10)-1,CEILING(J22,50)-1)</f>
-        <v>639</v>
+        <v>339</v>
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">K22-F22</f>
-        <v>254.41</v>
+        <v>155</v>
       </c>
       <c r="M22" s="11" t="n">
         <f aca="false">IF(K22=0,"",L22/K22)</f>
-        <v>0.398137715179969</v>
+        <v>0.457227138643068</v>
       </c>
       <c r="N22" s="11" t="n">
         <f aca="false">IF(F22=0,"",K22/F22-1)</f>
-        <v>0.661509659637536</v>
+        <v>0.842391304347826</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2013,48 +2193,48 @@
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>419.93</v>
+        <v>197.64</v>
       </c>
       <c r="G23" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F23,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H23" s="7"/>
       <c r="I23" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F23,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">IF(H23="",MAX(F23*(1+G23),I23),F23*(1+H23))</f>
-        <v>692.8845</v>
+        <v>355.752</v>
       </c>
       <c r="K23" s="10" t="n">
         <f aca="false">IF(J23&lt;1000,CEILING(J23,10)-1,CEILING(J23,50)-1)</f>
-        <v>699</v>
+        <v>359</v>
       </c>
       <c r="L23" s="9" t="n">
         <f aca="false">K23-F23</f>
-        <v>279.07</v>
+        <v>161.36</v>
       </c>
       <c r="M23" s="11" t="n">
         <f aca="false">IF(K23=0,"",L23/K23)</f>
-        <v>0.399241773962804</v>
+        <v>0.449470752089137</v>
       </c>
       <c r="N23" s="11" t="n">
         <f aca="false">IF(F23=0,"",K23/F23-1)</f>
-        <v>0.66456314147596</v>
+        <v>0.816433920259057</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2062,48 +2242,48 @@
         <v>20</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>525.56</v>
+        <v>275.63</v>
       </c>
       <c r="G24" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F24,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H24" s="7"/>
       <c r="I24" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F24,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J24" s="9" t="n">
         <f aca="false">IF(H24="",MAX(F24*(1+G24),I24),F24*(1+H24))</f>
-        <v>867.174</v>
+        <v>496.134</v>
       </c>
       <c r="K24" s="10" t="n">
         <f aca="false">IF(J24&lt;1000,CEILING(J24,10)-1,CEILING(J24,50)-1)</f>
-        <v>869</v>
+        <v>499</v>
       </c>
       <c r="L24" s="9" t="n">
         <f aca="false">K24-F24</f>
-        <v>343.44</v>
+        <v>223.37</v>
       </c>
       <c r="M24" s="11" t="n">
         <f aca="false">IF(K24=0,"",L24/K24)</f>
-        <v>0.395212888377445</v>
+        <v>0.447635270541082</v>
       </c>
       <c r="N24" s="11" t="n">
         <f aca="false">IF(F24=0,"",K24/F24-1)</f>
-        <v>0.653474389222924</v>
+        <v>0.810397997315242</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2111,19 +2291,19 @@
         <v>21</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>550.83</v>
+        <v>325.16</v>
       </c>
       <c r="G25" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F25,Reglas!$A$5:$A$8,1))</f>
@@ -2136,23 +2316,23 @@
       </c>
       <c r="J25" s="9" t="n">
         <f aca="false">IF(H25="",MAX(F25*(1+G25),I25),F25*(1+H25))</f>
-        <v>908.8695</v>
+        <v>540</v>
       </c>
       <c r="K25" s="10" t="n">
         <f aca="false">IF(J25&lt;1000,CEILING(J25,10)-1,CEILING(J25,50)-1)</f>
-        <v>909</v>
+        <v>539</v>
       </c>
       <c r="L25" s="9" t="n">
         <f aca="false">K25-F25</f>
-        <v>358.17</v>
+        <v>213.84</v>
       </c>
       <c r="M25" s="11" t="n">
         <f aca="false">IF(K25=0,"",L25/K25)</f>
-        <v>0.394026402640264</v>
+        <v>0.396734693877551</v>
       </c>
       <c r="N25" s="11" t="n">
         <f aca="false">IF(F25=0,"",K25/F25-1)</f>
-        <v>0.650236915200697</v>
+        <v>0.657645466847091</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2160,48 +2340,48 @@
         <v>22</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>950.19</v>
+        <v>359.45</v>
       </c>
       <c r="G26" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F26,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H26" s="7"/>
       <c r="I26" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F26,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J26" s="9" t="n">
         <f aca="false">IF(H26="",MAX(F26*(1+G26),I26),F26*(1+H26))</f>
-        <v>1472.7945</v>
+        <v>593.0925</v>
       </c>
       <c r="K26" s="10" t="n">
         <f aca="false">IF(J26&lt;1000,CEILING(J26,10)-1,CEILING(J26,50)-1)</f>
-        <v>1499</v>
+        <v>599</v>
       </c>
       <c r="L26" s="9" t="n">
         <f aca="false">K26-F26</f>
-        <v>548.81</v>
+        <v>239.55</v>
       </c>
       <c r="M26" s="11" t="n">
         <f aca="false">IF(K26=0,"",L26/K26)</f>
-        <v>0.366117411607739</v>
+        <v>0.39991652754591</v>
       </c>
       <c r="N26" s="11" t="n">
         <f aca="false">IF(F26=0,"",K26/F26-1)</f>
-        <v>0.577579220997906</v>
+        <v>0.666434830991793</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2209,48 +2389,48 @@
         <v>23</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>978.67</v>
+        <v>362.45</v>
       </c>
       <c r="G27" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F27,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H27" s="7"/>
       <c r="I27" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F27,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J27" s="9" t="n">
         <f aca="false">IF(H27="",MAX(F27*(1+G27),I27),F27*(1+H27))</f>
-        <v>1516.9385</v>
+        <v>598.0425</v>
       </c>
       <c r="K27" s="10" t="n">
         <f aca="false">IF(J27&lt;1000,CEILING(J27,10)-1,CEILING(J27,50)-1)</f>
-        <v>1549</v>
+        <v>599</v>
       </c>
       <c r="L27" s="9" t="n">
         <f aca="false">K27-F27</f>
-        <v>570.33</v>
+        <v>236.55</v>
       </c>
       <c r="M27" s="11" t="n">
         <f aca="false">IF(K27=0,"",L27/K27)</f>
-        <v>0.368192382182053</v>
+        <v>0.394908180300501</v>
       </c>
       <c r="N27" s="11" t="n">
         <f aca="false">IF(F27=0,"",K27/F27-1)</f>
-        <v>0.582760276702055</v>
+        <v>0.652641743688785</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2258,48 +2438,48 @@
         <v>24</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="E28" s="4" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>1608.09</v>
+        <v>487.77</v>
       </c>
       <c r="G28" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F28,Reglas!$A$5:$A$8,1))</f>
-        <v>0.45</v>
+        <v>0.65</v>
       </c>
       <c r="H28" s="7"/>
       <c r="I28" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F28,Reglas!$A$5:$A$8,1))</f>
-        <v>1860</v>
+        <v>540</v>
       </c>
       <c r="J28" s="9" t="n">
         <f aca="false">IF(H28="",MAX(F28*(1+G28),I28),F28*(1+H28))</f>
-        <v>2331.7305</v>
+        <v>804.8205</v>
       </c>
       <c r="K28" s="10" t="n">
         <f aca="false">IF(J28&lt;1000,CEILING(J28,10)-1,CEILING(J28,50)-1)</f>
-        <v>2349</v>
+        <v>809</v>
       </c>
       <c r="L28" s="9" t="n">
         <f aca="false">K28-F28</f>
-        <v>740.91</v>
+        <v>321.23</v>
       </c>
       <c r="M28" s="11" t="n">
         <f aca="false">IF(K28=0,"",L28/K28)</f>
-        <v>0.315415070242656</v>
+        <v>0.397070457354759</v>
       </c>
       <c r="N28" s="11" t="n">
         <f aca="false">IF(F28=0,"",K28/F28-1)</f>
-        <v>0.460739137734828</v>
+        <v>0.658568587654017</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2307,48 +2487,48 @@
         <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>1645.59</v>
+        <v>492.72</v>
       </c>
       <c r="G29" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F29,Reglas!$A$5:$A$8,1))</f>
-        <v>0.45</v>
+        <v>0.65</v>
       </c>
       <c r="H29" s="7"/>
       <c r="I29" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F29,Reglas!$A$5:$A$8,1))</f>
-        <v>1860</v>
+        <v>540</v>
       </c>
       <c r="J29" s="9" t="n">
         <f aca="false">IF(H29="",MAX(F29*(1+G29),I29),F29*(1+H29))</f>
-        <v>2386.1055</v>
+        <v>812.988</v>
       </c>
       <c r="K29" s="10" t="n">
         <f aca="false">IF(J29&lt;1000,CEILING(J29,10)-1,CEILING(J29,50)-1)</f>
-        <v>2399</v>
+        <v>819</v>
       </c>
       <c r="L29" s="9" t="n">
         <f aca="false">K29-F29</f>
-        <v>753.41</v>
+        <v>326.28</v>
       </c>
       <c r="M29" s="11" t="n">
         <f aca="false">IF(K29=0,"",L29/K29)</f>
-        <v>0.314051688203418</v>
+        <v>0.398388278388278</v>
       </c>
       <c r="N29" s="11" t="n">
         <f aca="false">IF(F29=0,"",K29/F29-1)</f>
-        <v>0.457835791418276</v>
+        <v>0.662201656113005</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2356,19 +2536,19 @@
         <v>26</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>321.42</v>
+        <v>515.85</v>
       </c>
       <c r="G30" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F30,Reglas!$A$5:$A$8,1))</f>
@@ -2381,23 +2561,23 @@
       </c>
       <c r="J30" s="9" t="n">
         <f aca="false">IF(H30="",MAX(F30*(1+G30),I30),F30*(1+H30))</f>
-        <v>540</v>
+        <v>851.1525</v>
       </c>
       <c r="K30" s="10" t="n">
         <f aca="false">IF(J30&lt;1000,CEILING(J30,10)-1,CEILING(J30,50)-1)</f>
-        <v>539</v>
+        <v>859</v>
       </c>
       <c r="L30" s="9" t="n">
         <f aca="false">K30-F30</f>
-        <v>217.58</v>
+        <v>343.15</v>
       </c>
       <c r="M30" s="11" t="n">
         <f aca="false">IF(K30=0,"",L30/K30)</f>
-        <v>0.403673469387755</v>
+        <v>0.399476135040745</v>
       </c>
       <c r="N30" s="11" t="n">
         <f aca="false">IF(F30=0,"",K30/F30-1)</f>
-        <v>0.676933607118412</v>
+        <v>0.665212755646021</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2405,19 +2585,19 @@
         <v>27</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>321.42</v>
+        <v>558.88</v>
       </c>
       <c r="G31" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F31,Reglas!$A$5:$A$8,1))</f>
@@ -2430,23 +2610,23 @@
       </c>
       <c r="J31" s="9" t="n">
         <f aca="false">IF(H31="",MAX(F31*(1+G31),I31),F31*(1+H31))</f>
-        <v>540</v>
+        <v>922.152</v>
       </c>
       <c r="K31" s="10" t="n">
         <f aca="false">IF(J31&lt;1000,CEILING(J31,10)-1,CEILING(J31,50)-1)</f>
-        <v>539</v>
+        <v>929</v>
       </c>
       <c r="L31" s="9" t="n">
         <f aca="false">K31-F31</f>
-        <v>217.58</v>
+        <v>370.12</v>
       </c>
       <c r="M31" s="11" t="n">
         <f aca="false">IF(K31=0,"",L31/K31)</f>
-        <v>0.403673469387755</v>
+        <v>0.398406889128095</v>
       </c>
       <c r="N31" s="11" t="n">
         <f aca="false">IF(F31=0,"",K31/F31-1)</f>
-        <v>0.676933607118412</v>
+        <v>0.662253077583739</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2454,19 +2634,19 @@
         <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="F32" s="5" t="n">
-        <v>823.36</v>
+        <v>705.08</v>
       </c>
       <c r="G32" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F32,Reglas!$A$5:$A$8,1))</f>
@@ -2479,23 +2659,23 @@
       </c>
       <c r="J32" s="9" t="n">
         <f aca="false">IF(H32="",MAX(F32*(1+G32),I32),F32*(1+H32))</f>
-        <v>1276.208</v>
+        <v>1155</v>
       </c>
       <c r="K32" s="10" t="n">
         <f aca="false">IF(J32&lt;1000,CEILING(J32,10)-1,CEILING(J32,50)-1)</f>
-        <v>1299</v>
+        <v>1199</v>
       </c>
       <c r="L32" s="9" t="n">
         <f aca="false">K32-F32</f>
-        <v>475.64</v>
+        <v>493.92</v>
       </c>
       <c r="M32" s="11" t="n">
         <f aca="false">IF(K32=0,"",L32/K32)</f>
-        <v>0.366158583525789</v>
+        <v>0.411943286071726</v>
       </c>
       <c r="N32" s="11" t="n">
         <f aca="false">IF(F32=0,"",K32/F32-1)</f>
-        <v>0.577681694520016</v>
+        <v>0.700516253474783</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2503,48 +2683,48 @@
         <v>29</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>177.68</v>
+        <v>821.52</v>
       </c>
       <c r="G33" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F33,Reglas!$A$5:$A$8,1))</f>
-        <v>0.8</v>
+        <v>0.55</v>
       </c>
       <c r="H33" s="7"/>
       <c r="I33" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F33,Reglas!$A$5:$A$8,1))</f>
-        <v>0</v>
+        <v>1155</v>
       </c>
       <c r="J33" s="9" t="n">
         <f aca="false">IF(H33="",MAX(F33*(1+G33),I33),F33*(1+H33))</f>
-        <v>319.824</v>
+        <v>1273.356</v>
       </c>
       <c r="K33" s="10" t="n">
         <f aca="false">IF(J33&lt;1000,CEILING(J33,10)-1,CEILING(J33,50)-1)</f>
-        <v>319</v>
+        <v>1299</v>
       </c>
       <c r="L33" s="9" t="n">
         <f aca="false">K33-F33</f>
-        <v>141.32</v>
+        <v>477.48</v>
       </c>
       <c r="M33" s="11" t="n">
         <f aca="false">IF(K33=0,"",L33/K33)</f>
-        <v>0.443009404388715</v>
+        <v>0.367575057736721</v>
       </c>
       <c r="N33" s="11" t="n">
         <f aca="false">IF(F33=0,"",K33/F33-1)</f>
-        <v>0.795362449347141</v>
+        <v>0.581215308209173</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2552,48 +2732,48 @@
         <v>30</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>305.32</v>
+        <v>150.28</v>
       </c>
       <c r="G34" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F34,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H34" s="7"/>
       <c r="I34" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F34,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J34" s="9" t="n">
         <f aca="false">IF(H34="",MAX(F34*(1+G34),I34),F34*(1+H34))</f>
-        <v>540</v>
+        <v>270.504</v>
       </c>
       <c r="K34" s="10" t="n">
         <f aca="false">IF(J34&lt;1000,CEILING(J34,10)-1,CEILING(J34,50)-1)</f>
-        <v>539</v>
+        <v>279</v>
       </c>
       <c r="L34" s="9" t="n">
         <f aca="false">K34-F34</f>
-        <v>233.68</v>
+        <v>128.72</v>
       </c>
       <c r="M34" s="11" t="n">
         <f aca="false">IF(K34=0,"",L34/K34)</f>
-        <v>0.433543599257885</v>
+        <v>0.461362007168459</v>
       </c>
       <c r="N34" s="11" t="n">
         <f aca="false">IF(F34=0,"",K34/F34-1)</f>
-        <v>0.765360932791825</v>
+        <v>0.856534468991216</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2601,48 +2781,48 @@
         <v>31</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C35" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D35" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>86</v>
-      </c>
       <c r="F35" s="5" t="n">
-        <v>423.82</v>
+        <v>174.54</v>
       </c>
       <c r="G35" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F35,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F35,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J35" s="9" t="n">
         <f aca="false">IF(H35="",MAX(F35*(1+G35),I35),F35*(1+H35))</f>
-        <v>699.303</v>
+        <v>314.172</v>
       </c>
       <c r="K35" s="10" t="n">
         <f aca="false">IF(J35&lt;1000,CEILING(J35,10)-1,CEILING(J35,50)-1)</f>
-        <v>699</v>
+        <v>319</v>
       </c>
       <c r="L35" s="9" t="n">
         <f aca="false">K35-F35</f>
-        <v>275.18</v>
+        <v>144.46</v>
       </c>
       <c r="M35" s="11" t="n">
         <f aca="false">IF(K35=0,"",L35/K35)</f>
-        <v>0.393676680972818</v>
+        <v>0.452852664576803</v>
       </c>
       <c r="N35" s="11" t="n">
         <f aca="false">IF(F35=0,"",K35/F35-1)</f>
-        <v>0.649285073852107</v>
+        <v>0.827661281081701</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2650,19 +2830,19 @@
         <v>32</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>436.23</v>
+        <v>319.2</v>
       </c>
       <c r="G36" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F36,Reglas!$A$5:$A$8,1))</f>
@@ -2675,23 +2855,23 @@
       </c>
       <c r="J36" s="9" t="n">
         <f aca="false">IF(H36="",MAX(F36*(1+G36),I36),F36*(1+H36))</f>
-        <v>719.7795</v>
+        <v>540</v>
       </c>
       <c r="K36" s="10" t="n">
         <f aca="false">IF(J36&lt;1000,CEILING(J36,10)-1,CEILING(J36,50)-1)</f>
-        <v>719</v>
+        <v>539</v>
       </c>
       <c r="L36" s="9" t="n">
         <f aca="false">K36-F36</f>
-        <v>282.77</v>
+        <v>219.8</v>
       </c>
       <c r="M36" s="11" t="n">
         <f aca="false">IF(K36=0,"",L36/K36)</f>
-        <v>0.393282336578581</v>
+        <v>0.407792207792208</v>
       </c>
       <c r="N36" s="11" t="n">
         <f aca="false">IF(F36=0,"",K36/F36-1)</f>
-        <v>0.648213098594778</v>
+        <v>0.68859649122807</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2699,19 +2879,19 @@
         <v>33</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>509.54</v>
+        <v>324.7</v>
       </c>
       <c r="G37" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F37,Reglas!$A$5:$A$8,1))</f>
@@ -2724,23 +2904,23 @@
       </c>
       <c r="J37" s="9" t="n">
         <f aca="false">IF(H37="",MAX(F37*(1+G37),I37),F37*(1+H37))</f>
-        <v>840.741</v>
+        <v>540</v>
       </c>
       <c r="K37" s="10" t="n">
         <f aca="false">IF(J37&lt;1000,CEILING(J37,10)-1,CEILING(J37,50)-1)</f>
-        <v>849</v>
+        <v>539</v>
       </c>
       <c r="L37" s="9" t="n">
         <f aca="false">K37-F37</f>
-        <v>339.46</v>
+        <v>214.3</v>
       </c>
       <c r="M37" s="11" t="n">
         <f aca="false">IF(K37=0,"",L37/K37)</f>
-        <v>0.399835100117786</v>
+        <v>0.397588126159555</v>
       </c>
       <c r="N37" s="11" t="n">
         <f aca="false">IF(F37=0,"",K37/F37-1)</f>
-        <v>0.66620873729246</v>
+        <v>0.659993840468125</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2748,48 +2928,48 @@
         <v>34</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>145.06</v>
+        <v>401.75</v>
       </c>
       <c r="G38" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F38,Reglas!$A$5:$A$8,1))</f>
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="H38" s="7"/>
       <c r="I38" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F38,Reglas!$A$5:$A$8,1))</f>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="J38" s="9" t="n">
         <f aca="false">IF(H38="",MAX(F38*(1+G38),I38),F38*(1+H38))</f>
-        <v>261.108</v>
+        <v>662.8875</v>
       </c>
       <c r="K38" s="10" t="n">
         <f aca="false">IF(J38&lt;1000,CEILING(J38,10)-1,CEILING(J38,50)-1)</f>
-        <v>269</v>
+        <v>669</v>
       </c>
       <c r="L38" s="9" t="n">
         <f aca="false">K38-F38</f>
-        <v>123.94</v>
+        <v>267.25</v>
       </c>
       <c r="M38" s="11" t="n">
         <f aca="false">IF(K38=0,"",L38/K38)</f>
-        <v>0.460743494423792</v>
+        <v>0.399476831091181</v>
       </c>
       <c r="N38" s="11" t="n">
         <f aca="false">IF(F38=0,"",K38/F38-1)</f>
-        <v>0.854405073762581</v>
+        <v>0.665214685749844</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2797,48 +2977,48 @@
         <v>35</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>157.44</v>
+        <v>422.36</v>
       </c>
       <c r="G39" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F39,Reglas!$A$5:$A$8,1))</f>
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="H39" s="7"/>
       <c r="I39" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F39,Reglas!$A$5:$A$8,1))</f>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="J39" s="9" t="n">
         <f aca="false">IF(H39="",MAX(F39*(1+G39),I39),F39*(1+H39))</f>
-        <v>283.392</v>
+        <v>696.894</v>
       </c>
       <c r="K39" s="10" t="n">
         <f aca="false">IF(J39&lt;1000,CEILING(J39,10)-1,CEILING(J39,50)-1)</f>
-        <v>289</v>
+        <v>699</v>
       </c>
       <c r="L39" s="9" t="n">
         <f aca="false">K39-F39</f>
-        <v>131.56</v>
+        <v>276.64</v>
       </c>
       <c r="M39" s="11" t="n">
         <f aca="false">IF(K39=0,"",L39/K39)</f>
-        <v>0.45522491349481</v>
+        <v>0.395765379113019</v>
       </c>
       <c r="N39" s="11" t="n">
         <f aca="false">IF(F39=0,"",K39/F39-1)</f>
-        <v>0.835619918699187</v>
+        <v>0.654986267638981</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2846,19 +3026,19 @@
         <v>36</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>327.59</v>
+        <v>427.15</v>
       </c>
       <c r="G40" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F40,Reglas!$A$5:$A$8,1))</f>
@@ -2871,23 +3051,23 @@
       </c>
       <c r="J40" s="9" t="n">
         <f aca="false">IF(H40="",MAX(F40*(1+G40),I40),F40*(1+H40))</f>
-        <v>540.5235</v>
+        <v>704.7975</v>
       </c>
       <c r="K40" s="10" t="n">
         <f aca="false">IF(J40&lt;1000,CEILING(J40,10)-1,CEILING(J40,50)-1)</f>
-        <v>549</v>
+        <v>709</v>
       </c>
       <c r="L40" s="9" t="n">
         <f aca="false">K40-F40</f>
-        <v>221.41</v>
+        <v>281.85</v>
       </c>
       <c r="M40" s="11" t="n">
         <f aca="false">IF(K40=0,"",L40/K40)</f>
-        <v>0.403296903460838</v>
+        <v>0.3975317348378</v>
       </c>
       <c r="N40" s="11" t="n">
         <f aca="false">IF(F40=0,"",K40/F40-1)</f>
-        <v>0.675875331969841</v>
+        <v>0.659838464239729</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2895,19 +3075,19 @@
         <v>37</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>100</v>
-      </c>
       <c r="F41" s="5" t="n">
-        <v>416.39</v>
+        <v>532.85</v>
       </c>
       <c r="G41" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F41,Reglas!$A$5:$A$8,1))</f>
@@ -2920,23 +3100,23 @@
       </c>
       <c r="J41" s="9" t="n">
         <f aca="false">IF(H41="",MAX(F41*(1+G41),I41),F41*(1+H41))</f>
-        <v>687.0435</v>
+        <v>879.2025</v>
       </c>
       <c r="K41" s="10" t="n">
         <f aca="false">IF(J41&lt;1000,CEILING(J41,10)-1,CEILING(J41,50)-1)</f>
-        <v>689</v>
+        <v>879</v>
       </c>
       <c r="L41" s="9" t="n">
         <f aca="false">K41-F41</f>
-        <v>272.61</v>
+        <v>346.15</v>
       </c>
       <c r="M41" s="11" t="n">
         <f aca="false">IF(K41=0,"",L41/K41)</f>
-        <v>0.395660377358491</v>
+        <v>0.393799772468714</v>
       </c>
       <c r="N41" s="11" t="n">
         <f aca="false">IF(F41=0,"",K41/F41-1)</f>
-        <v>0.654698719950047</v>
+        <v>0.649619968096087</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2944,19 +3124,19 @@
         <v>38</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>496.84</v>
+        <v>377.88</v>
       </c>
       <c r="G42" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F42,Reglas!$A$5:$A$8,1))</f>
@@ -2969,23 +3149,23 @@
       </c>
       <c r="J42" s="9" t="n">
         <f aca="false">IF(H42="",MAX(F42*(1+G42),I42),F42*(1+H42))</f>
-        <v>819.786</v>
+        <v>623.502</v>
       </c>
       <c r="K42" s="10" t="n">
         <f aca="false">IF(J42&lt;1000,CEILING(J42,10)-1,CEILING(J42,50)-1)</f>
-        <v>819</v>
+        <v>629</v>
       </c>
       <c r="L42" s="9" t="n">
         <f aca="false">K42-F42</f>
-        <v>322.16</v>
+        <v>251.12</v>
       </c>
       <c r="M42" s="11" t="n">
         <f aca="false">IF(K42=0,"",L42/K42)</f>
-        <v>0.393357753357753</v>
+        <v>0.399236883942766</v>
       </c>
       <c r="N42" s="11" t="n">
         <f aca="false">IF(F42=0,"",K42/F42-1)</f>
-        <v>0.648418001771194</v>
+        <v>0.664549592463216</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2993,82 +3173,1552 @@
         <v>39</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>1405.86</v>
+        <v>737.5</v>
       </c>
       <c r="G43" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F43,Reglas!$A$5:$A$8,1))</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="H43" s="7"/>
       <c r="I43" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F43,Reglas!$A$5:$A$8,1))</f>
-        <v>1860</v>
+        <v>1155</v>
       </c>
       <c r="J43" s="9" t="n">
         <f aca="false">IF(H43="",MAX(F43*(1+G43),I43),F43*(1+H43))</f>
-        <v>2038.497</v>
+        <v>1155</v>
       </c>
       <c r="K43" s="10" t="n">
         <f aca="false">IF(J43&lt;1000,CEILING(J43,10)-1,CEILING(J43,50)-1)</f>
-        <v>2049</v>
+        <v>1199</v>
       </c>
       <c r="L43" s="9" t="n">
         <f aca="false">K43-F43</f>
-        <v>643.14</v>
+        <v>461.5</v>
       </c>
       <c r="M43" s="11" t="n">
         <f aca="false">IF(K43=0,"",L43/K43)</f>
-        <v>0.313879941434846</v>
+        <v>0.384904086738949</v>
       </c>
       <c r="N43" s="11" t="n">
         <f aca="false">IF(F43=0,"",K43/F43-1)</f>
+        <v>0.625762711864407</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>866.93</v>
+      </c>
+      <c r="G44" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F44,Reglas!$A$5:$A$8,1))</f>
+        <v>0.55</v>
+      </c>
+      <c r="H44" s="7"/>
+      <c r="I44" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F44,Reglas!$A$5:$A$8,1))</f>
+        <v>1155</v>
+      </c>
+      <c r="J44" s="9" t="n">
+        <f aca="false">IF(H44="",MAX(F44*(1+G44),I44),F44*(1+H44))</f>
+        <v>1343.7415</v>
+      </c>
+      <c r="K44" s="10" t="n">
+        <f aca="false">IF(J44&lt;1000,CEILING(J44,10)-1,CEILING(J44,50)-1)</f>
+        <v>1349</v>
+      </c>
+      <c r="L44" s="9" t="n">
+        <f aca="false">K44-F44</f>
+        <v>482.07</v>
+      </c>
+      <c r="M44" s="11" t="n">
+        <f aca="false">IF(K44=0,"",L44/K44)</f>
+        <v>0.357353595255745</v>
+      </c>
+      <c r="N44" s="11" t="n">
+        <f aca="false">IF(F44=0,"",K44/F44-1)</f>
+        <v>0.556065656973458</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>901.39</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F45,Reglas!$A$5:$A$8,1))</f>
+        <v>0.55</v>
+      </c>
+      <c r="H45" s="7"/>
+      <c r="I45" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F45,Reglas!$A$5:$A$8,1))</f>
+        <v>1155</v>
+      </c>
+      <c r="J45" s="9" t="n">
+        <f aca="false">IF(H45="",MAX(F45*(1+G45),I45),F45*(1+H45))</f>
+        <v>1397.1545</v>
+      </c>
+      <c r="K45" s="10" t="n">
+        <f aca="false">IF(J45&lt;1000,CEILING(J45,10)-1,CEILING(J45,50)-1)</f>
+        <v>1399</v>
+      </c>
+      <c r="L45" s="9" t="n">
+        <f aca="false">K45-F45</f>
+        <v>497.61</v>
+      </c>
+      <c r="M45" s="11" t="n">
+        <f aca="false">IF(K45=0,"",L45/K45)</f>
+        <v>0.355689778413152</v>
+      </c>
+      <c r="N45" s="11" t="n">
+        <f aca="false">IF(F45=0,"",K45/F45-1)</f>
+        <v>0.552047393470085</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>1012.41</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F46,Reglas!$A$5:$A$8,1))</f>
+        <v>0.55</v>
+      </c>
+      <c r="H46" s="7"/>
+      <c r="I46" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F46,Reglas!$A$5:$A$8,1))</f>
+        <v>1155</v>
+      </c>
+      <c r="J46" s="9" t="n">
+        <f aca="false">IF(H46="",MAX(F46*(1+G46),I46),F46*(1+H46))</f>
+        <v>1569.2355</v>
+      </c>
+      <c r="K46" s="10" t="n">
+        <f aca="false">IF(J46&lt;1000,CEILING(J46,10)-1,CEILING(J46,50)-1)</f>
+        <v>1599</v>
+      </c>
+      <c r="L46" s="9" t="n">
+        <f aca="false">K46-F46</f>
+        <v>586.59</v>
+      </c>
+      <c r="M46" s="11" t="n">
+        <f aca="false">IF(K46=0,"",L46/K46)</f>
+        <v>0.366848030018762</v>
+      </c>
+      <c r="N46" s="11" t="n">
+        <f aca="false">IF(F46=0,"",K46/F46-1)</f>
+        <v>0.57939965033929</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>1047.3</v>
+      </c>
+      <c r="G47" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F47,Reglas!$A$5:$A$8,1))</f>
+        <v>0.55</v>
+      </c>
+      <c r="H47" s="7"/>
+      <c r="I47" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F47,Reglas!$A$5:$A$8,1))</f>
+        <v>1155</v>
+      </c>
+      <c r="J47" s="9" t="n">
+        <f aca="false">IF(H47="",MAX(F47*(1+G47),I47),F47*(1+H47))</f>
+        <v>1623.315</v>
+      </c>
+      <c r="K47" s="10" t="n">
+        <f aca="false">IF(J47&lt;1000,CEILING(J47,10)-1,CEILING(J47,50)-1)</f>
+        <v>1649</v>
+      </c>
+      <c r="L47" s="9" t="n">
+        <f aca="false">K47-F47</f>
+        <v>601.7</v>
+      </c>
+      <c r="M47" s="11" t="n">
+        <f aca="false">IF(K47=0,"",L47/K47)</f>
+        <v>0.364887810794421</v>
+      </c>
+      <c r="N47" s="11" t="n">
+        <f aca="false">IF(F47=0,"",K47/F47-1)</f>
+        <v>0.574524968967822</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>1275.69</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F48,Reglas!$A$5:$A$8,1))</f>
+        <v>0.45</v>
+      </c>
+      <c r="H48" s="7"/>
+      <c r="I48" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F48,Reglas!$A$5:$A$8,1))</f>
+        <v>1860</v>
+      </c>
+      <c r="J48" s="9" t="n">
+        <f aca="false">IF(H48="",MAX(F48*(1+G48),I48),F48*(1+H48))</f>
+        <v>1860</v>
+      </c>
+      <c r="K48" s="10" t="n">
+        <f aca="false">IF(J48&lt;1000,CEILING(J48,10)-1,CEILING(J48,50)-1)</f>
+        <v>1899</v>
+      </c>
+      <c r="L48" s="9" t="n">
+        <f aca="false">K48-F48</f>
+        <v>623.31</v>
+      </c>
+      <c r="M48" s="11" t="n">
+        <f aca="false">IF(K48=0,"",L48/K48)</f>
+        <v>0.328230647709321</v>
+      </c>
+      <c r="N48" s="11" t="n">
+        <f aca="false">IF(F48=0,"",K48/F48-1)</f>
+        <v>0.48860616607483</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>2411.07</v>
+      </c>
+      <c r="G49" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F49,Reglas!$A$5:$A$8,1))</f>
+        <v>0.45</v>
+      </c>
+      <c r="H49" s="7"/>
+      <c r="I49" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F49,Reglas!$A$5:$A$8,1))</f>
+        <v>1860</v>
+      </c>
+      <c r="J49" s="9" t="n">
+        <f aca="false">IF(H49="",MAX(F49*(1+G49),I49),F49*(1+H49))</f>
+        <v>3496.0515</v>
+      </c>
+      <c r="K49" s="10" t="n">
+        <f aca="false">IF(J49&lt;1000,CEILING(J49,10)-1,CEILING(J49,50)-1)</f>
+        <v>3499</v>
+      </c>
+      <c r="L49" s="9" t="n">
+        <f aca="false">K49-F49</f>
+        <v>1087.93</v>
+      </c>
+      <c r="M49" s="11" t="n">
+        <f aca="false">IF(K49=0,"",L49/K49)</f>
+        <v>0.3109259788511</v>
+      </c>
+      <c r="N49" s="11" t="n">
+        <f aca="false">IF(F49=0,"",K49/F49-1)</f>
+        <v>0.45122290103564</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>362.5</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F50,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H50" s="7"/>
+      <c r="I50" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F50,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J50" s="9" t="n">
+        <f aca="false">IF(H50="",MAX(F50*(1+G50),I50),F50*(1+H50))</f>
+        <v>598.125</v>
+      </c>
+      <c r="K50" s="10" t="n">
+        <f aca="false">IF(J50&lt;1000,CEILING(J50,10)-1,CEILING(J50,50)-1)</f>
+        <v>599</v>
+      </c>
+      <c r="L50" s="9" t="n">
+        <f aca="false">K50-F50</f>
+        <v>236.5</v>
+      </c>
+      <c r="M50" s="11" t="n">
+        <f aca="false">IF(K50=0,"",L50/K50)</f>
+        <v>0.394824707846411</v>
+      </c>
+      <c r="N50" s="11" t="n">
+        <f aca="false">IF(F50=0,"",K50/F50-1)</f>
+        <v>0.652413793103448</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>384.06</v>
+      </c>
+      <c r="G51" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F51,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H51" s="7"/>
+      <c r="I51" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F51,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J51" s="9" t="n">
+        <f aca="false">IF(H51="",MAX(F51*(1+G51),I51),F51*(1+H51))</f>
+        <v>633.699</v>
+      </c>
+      <c r="K51" s="10" t="n">
+        <f aca="false">IF(J51&lt;1000,CEILING(J51,10)-1,CEILING(J51,50)-1)</f>
+        <v>639</v>
+      </c>
+      <c r="L51" s="9" t="n">
+        <f aca="false">K51-F51</f>
+        <v>254.94</v>
+      </c>
+      <c r="M51" s="11" t="n">
+        <f aca="false">IF(K51=0,"",L51/K51)</f>
+        <v>0.398967136150235</v>
+      </c>
+      <c r="N51" s="11" t="n">
+        <f aca="false">IF(F51=0,"",K51/F51-1)</f>
+        <v>0.663802530854554</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>384.59</v>
+      </c>
+      <c r="G52" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F52,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H52" s="7"/>
+      <c r="I52" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F52,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <f aca="false">IF(H52="",MAX(F52*(1+G52),I52),F52*(1+H52))</f>
+        <v>634.5735</v>
+      </c>
+      <c r="K52" s="10" t="n">
+        <f aca="false">IF(J52&lt;1000,CEILING(J52,10)-1,CEILING(J52,50)-1)</f>
+        <v>639</v>
+      </c>
+      <c r="L52" s="9" t="n">
+        <f aca="false">K52-F52</f>
+        <v>254.41</v>
+      </c>
+      <c r="M52" s="11" t="n">
+        <f aca="false">IF(K52=0,"",L52/K52)</f>
+        <v>0.398137715179969</v>
+      </c>
+      <c r="N52" s="11" t="n">
+        <f aca="false">IF(F52=0,"",K52/F52-1)</f>
+        <v>0.661509659637536</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>419.93</v>
+      </c>
+      <c r="G53" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F53,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H53" s="7"/>
+      <c r="I53" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F53,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J53" s="9" t="n">
+        <f aca="false">IF(H53="",MAX(F53*(1+G53),I53),F53*(1+H53))</f>
+        <v>692.8845</v>
+      </c>
+      <c r="K53" s="10" t="n">
+        <f aca="false">IF(J53&lt;1000,CEILING(J53,10)-1,CEILING(J53,50)-1)</f>
+        <v>699</v>
+      </c>
+      <c r="L53" s="9" t="n">
+        <f aca="false">K53-F53</f>
+        <v>279.07</v>
+      </c>
+      <c r="M53" s="11" t="n">
+        <f aca="false">IF(K53=0,"",L53/K53)</f>
+        <v>0.399241773962804</v>
+      </c>
+      <c r="N53" s="11" t="n">
+        <f aca="false">IF(F53=0,"",K53/F53-1)</f>
+        <v>0.66456314147596</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>525.56</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F54,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H54" s="7"/>
+      <c r="I54" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F54,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J54" s="9" t="n">
+        <f aca="false">IF(H54="",MAX(F54*(1+G54),I54),F54*(1+H54))</f>
+        <v>867.174</v>
+      </c>
+      <c r="K54" s="10" t="n">
+        <f aca="false">IF(J54&lt;1000,CEILING(J54,10)-1,CEILING(J54,50)-1)</f>
+        <v>869</v>
+      </c>
+      <c r="L54" s="9" t="n">
+        <f aca="false">K54-F54</f>
+        <v>343.44</v>
+      </c>
+      <c r="M54" s="11" t="n">
+        <f aca="false">IF(K54=0,"",L54/K54)</f>
+        <v>0.395212888377445</v>
+      </c>
+      <c r="N54" s="11" t="n">
+        <f aca="false">IF(F54=0,"",K54/F54-1)</f>
+        <v>0.653474389222924</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F55" s="5" t="n">
+        <v>550.83</v>
+      </c>
+      <c r="G55" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F55,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H55" s="7"/>
+      <c r="I55" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F55,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J55" s="9" t="n">
+        <f aca="false">IF(H55="",MAX(F55*(1+G55),I55),F55*(1+H55))</f>
+        <v>908.8695</v>
+      </c>
+      <c r="K55" s="10" t="n">
+        <f aca="false">IF(J55&lt;1000,CEILING(J55,10)-1,CEILING(J55,50)-1)</f>
+        <v>909</v>
+      </c>
+      <c r="L55" s="9" t="n">
+        <f aca="false">K55-F55</f>
+        <v>358.17</v>
+      </c>
+      <c r="M55" s="11" t="n">
+        <f aca="false">IF(K55=0,"",L55/K55)</f>
+        <v>0.394026402640264</v>
+      </c>
+      <c r="N55" s="11" t="n">
+        <f aca="false">IF(F55=0,"",K55/F55-1)</f>
+        <v>0.650236915200697</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>950.19</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F56,Reglas!$A$5:$A$8,1))</f>
+        <v>0.55</v>
+      </c>
+      <c r="H56" s="7"/>
+      <c r="I56" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F56,Reglas!$A$5:$A$8,1))</f>
+        <v>1155</v>
+      </c>
+      <c r="J56" s="9" t="n">
+        <f aca="false">IF(H56="",MAX(F56*(1+G56),I56),F56*(1+H56))</f>
+        <v>1472.7945</v>
+      </c>
+      <c r="K56" s="10" t="n">
+        <f aca="false">IF(J56&lt;1000,CEILING(J56,10)-1,CEILING(J56,50)-1)</f>
+        <v>1499</v>
+      </c>
+      <c r="L56" s="9" t="n">
+        <f aca="false">K56-F56</f>
+        <v>548.81</v>
+      </c>
+      <c r="M56" s="11" t="n">
+        <f aca="false">IF(K56=0,"",L56/K56)</f>
+        <v>0.366117411607739</v>
+      </c>
+      <c r="N56" s="11" t="n">
+        <f aca="false">IF(F56=0,"",K56/F56-1)</f>
+        <v>0.577579220997906</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F57" s="5" t="n">
+        <v>978.67</v>
+      </c>
+      <c r="G57" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F57,Reglas!$A$5:$A$8,1))</f>
+        <v>0.55</v>
+      </c>
+      <c r="H57" s="7"/>
+      <c r="I57" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F57,Reglas!$A$5:$A$8,1))</f>
+        <v>1155</v>
+      </c>
+      <c r="J57" s="9" t="n">
+        <f aca="false">IF(H57="",MAX(F57*(1+G57),I57),F57*(1+H57))</f>
+        <v>1516.9385</v>
+      </c>
+      <c r="K57" s="10" t="n">
+        <f aca="false">IF(J57&lt;1000,CEILING(J57,10)-1,CEILING(J57,50)-1)</f>
+        <v>1549</v>
+      </c>
+      <c r="L57" s="9" t="n">
+        <f aca="false">K57-F57</f>
+        <v>570.33</v>
+      </c>
+      <c r="M57" s="11" t="n">
+        <f aca="false">IF(K57=0,"",L57/K57)</f>
+        <v>0.368192382182053</v>
+      </c>
+      <c r="N57" s="11" t="n">
+        <f aca="false">IF(F57=0,"",K57/F57-1)</f>
+        <v>0.582760276702055</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F58" s="5" t="n">
+        <v>1608.09</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F58,Reglas!$A$5:$A$8,1))</f>
+        <v>0.45</v>
+      </c>
+      <c r="H58" s="7"/>
+      <c r="I58" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F58,Reglas!$A$5:$A$8,1))</f>
+        <v>1860</v>
+      </c>
+      <c r="J58" s="9" t="n">
+        <f aca="false">IF(H58="",MAX(F58*(1+G58),I58),F58*(1+H58))</f>
+        <v>2331.7305</v>
+      </c>
+      <c r="K58" s="10" t="n">
+        <f aca="false">IF(J58&lt;1000,CEILING(J58,10)-1,CEILING(J58,50)-1)</f>
+        <v>2349</v>
+      </c>
+      <c r="L58" s="9" t="n">
+        <f aca="false">K58-F58</f>
+        <v>740.91</v>
+      </c>
+      <c r="M58" s="11" t="n">
+        <f aca="false">IF(K58=0,"",L58/K58)</f>
+        <v>0.315415070242656</v>
+      </c>
+      <c r="N58" s="11" t="n">
+        <f aca="false">IF(F58=0,"",K58/F58-1)</f>
+        <v>0.460739137734828</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F59" s="5" t="n">
+        <v>1645.59</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F59,Reglas!$A$5:$A$8,1))</f>
+        <v>0.45</v>
+      </c>
+      <c r="H59" s="7"/>
+      <c r="I59" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F59,Reglas!$A$5:$A$8,1))</f>
+        <v>1860</v>
+      </c>
+      <c r="J59" s="9" t="n">
+        <f aca="false">IF(H59="",MAX(F59*(1+G59),I59),F59*(1+H59))</f>
+        <v>2386.1055</v>
+      </c>
+      <c r="K59" s="10" t="n">
+        <f aca="false">IF(J59&lt;1000,CEILING(J59,10)-1,CEILING(J59,50)-1)</f>
+        <v>2399</v>
+      </c>
+      <c r="L59" s="9" t="n">
+        <f aca="false">K59-F59</f>
+        <v>753.41</v>
+      </c>
+      <c r="M59" s="11" t="n">
+        <f aca="false">IF(K59=0,"",L59/K59)</f>
+        <v>0.314051688203418</v>
+      </c>
+      <c r="N59" s="11" t="n">
+        <f aca="false">IF(F59=0,"",K59/F59-1)</f>
+        <v>0.457835791418276</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F60" s="5" t="n">
+        <v>321.42</v>
+      </c>
+      <c r="G60" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F60,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H60" s="7"/>
+      <c r="I60" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F60,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J60" s="9" t="n">
+        <f aca="false">IF(H60="",MAX(F60*(1+G60),I60),F60*(1+H60))</f>
+        <v>540</v>
+      </c>
+      <c r="K60" s="10" t="n">
+        <f aca="false">IF(J60&lt;1000,CEILING(J60,10)-1,CEILING(J60,50)-1)</f>
+        <v>539</v>
+      </c>
+      <c r="L60" s="9" t="n">
+        <f aca="false">K60-F60</f>
+        <v>217.58</v>
+      </c>
+      <c r="M60" s="11" t="n">
+        <f aca="false">IF(K60=0,"",L60/K60)</f>
+        <v>0.403673469387755</v>
+      </c>
+      <c r="N60" s="11" t="n">
+        <f aca="false">IF(F60=0,"",K60/F60-1)</f>
+        <v>0.676933607118412</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F61" s="5" t="n">
+        <v>321.42</v>
+      </c>
+      <c r="G61" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F61,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H61" s="7"/>
+      <c r="I61" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F61,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J61" s="9" t="n">
+        <f aca="false">IF(H61="",MAX(F61*(1+G61),I61),F61*(1+H61))</f>
+        <v>540</v>
+      </c>
+      <c r="K61" s="10" t="n">
+        <f aca="false">IF(J61&lt;1000,CEILING(J61,10)-1,CEILING(J61,50)-1)</f>
+        <v>539</v>
+      </c>
+      <c r="L61" s="9" t="n">
+        <f aca="false">K61-F61</f>
+        <v>217.58</v>
+      </c>
+      <c r="M61" s="11" t="n">
+        <f aca="false">IF(K61=0,"",L61/K61)</f>
+        <v>0.403673469387755</v>
+      </c>
+      <c r="N61" s="11" t="n">
+        <f aca="false">IF(F61=0,"",K61/F61-1)</f>
+        <v>0.676933607118412</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F62" s="5" t="n">
+        <v>823.36</v>
+      </c>
+      <c r="G62" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F62,Reglas!$A$5:$A$8,1))</f>
+        <v>0.55</v>
+      </c>
+      <c r="H62" s="7"/>
+      <c r="I62" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F62,Reglas!$A$5:$A$8,1))</f>
+        <v>1155</v>
+      </c>
+      <c r="J62" s="9" t="n">
+        <f aca="false">IF(H62="",MAX(F62*(1+G62),I62),F62*(1+H62))</f>
+        <v>1276.208</v>
+      </c>
+      <c r="K62" s="10" t="n">
+        <f aca="false">IF(J62&lt;1000,CEILING(J62,10)-1,CEILING(J62,50)-1)</f>
+        <v>1299</v>
+      </c>
+      <c r="L62" s="9" t="n">
+        <f aca="false">K62-F62</f>
+        <v>475.64</v>
+      </c>
+      <c r="M62" s="11" t="n">
+        <f aca="false">IF(K62=0,"",L62/K62)</f>
+        <v>0.366158583525789</v>
+      </c>
+      <c r="N62" s="11" t="n">
+        <f aca="false">IF(F62=0,"",K62/F62-1)</f>
+        <v>0.577681694520016</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F63" s="5" t="n">
+        <v>177.68</v>
+      </c>
+      <c r="G63" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F63,Reglas!$A$5:$A$8,1))</f>
+        <v>0.8</v>
+      </c>
+      <c r="H63" s="7"/>
+      <c r="I63" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F63,Reglas!$A$5:$A$8,1))</f>
+        <v>0</v>
+      </c>
+      <c r="J63" s="9" t="n">
+        <f aca="false">IF(H63="",MAX(F63*(1+G63),I63),F63*(1+H63))</f>
+        <v>319.824</v>
+      </c>
+      <c r="K63" s="10" t="n">
+        <f aca="false">IF(J63&lt;1000,CEILING(J63,10)-1,CEILING(J63,50)-1)</f>
+        <v>319</v>
+      </c>
+      <c r="L63" s="9" t="n">
+        <f aca="false">K63-F63</f>
+        <v>141.32</v>
+      </c>
+      <c r="M63" s="11" t="n">
+        <f aca="false">IF(K63=0,"",L63/K63)</f>
+        <v>0.443009404388715</v>
+      </c>
+      <c r="N63" s="11" t="n">
+        <f aca="false">IF(F63=0,"",K63/F63-1)</f>
+        <v>0.795362449347141</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F64" s="5" t="n">
+        <v>305.32</v>
+      </c>
+      <c r="G64" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F64,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H64" s="7"/>
+      <c r="I64" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F64,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J64" s="9" t="n">
+        <f aca="false">IF(H64="",MAX(F64*(1+G64),I64),F64*(1+H64))</f>
+        <v>540</v>
+      </c>
+      <c r="K64" s="10" t="n">
+        <f aca="false">IF(J64&lt;1000,CEILING(J64,10)-1,CEILING(J64,50)-1)</f>
+        <v>539</v>
+      </c>
+      <c r="L64" s="9" t="n">
+        <f aca="false">K64-F64</f>
+        <v>233.68</v>
+      </c>
+      <c r="M64" s="11" t="n">
+        <f aca="false">IF(K64=0,"",L64/K64)</f>
+        <v>0.433543599257885</v>
+      </c>
+      <c r="N64" s="11" t="n">
+        <f aca="false">IF(F64=0,"",K64/F64-1)</f>
+        <v>0.765360932791825</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="F65" s="5" t="n">
+        <v>423.82</v>
+      </c>
+      <c r="G65" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F65,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H65" s="7"/>
+      <c r="I65" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F65,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J65" s="9" t="n">
+        <f aca="false">IF(H65="",MAX(F65*(1+G65),I65),F65*(1+H65))</f>
+        <v>699.303</v>
+      </c>
+      <c r="K65" s="10" t="n">
+        <f aca="false">IF(J65&lt;1000,CEILING(J65,10)-1,CEILING(J65,50)-1)</f>
+        <v>699</v>
+      </c>
+      <c r="L65" s="9" t="n">
+        <f aca="false">K65-F65</f>
+        <v>275.18</v>
+      </c>
+      <c r="M65" s="11" t="n">
+        <f aca="false">IF(K65=0,"",L65/K65)</f>
+        <v>0.393676680972818</v>
+      </c>
+      <c r="N65" s="11" t="n">
+        <f aca="false">IF(F65=0,"",K65/F65-1)</f>
+        <v>0.649285073852107</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F66" s="5" t="n">
+        <v>436.23</v>
+      </c>
+      <c r="G66" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F66,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H66" s="7"/>
+      <c r="I66" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F66,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J66" s="9" t="n">
+        <f aca="false">IF(H66="",MAX(F66*(1+G66),I66),F66*(1+H66))</f>
+        <v>719.7795</v>
+      </c>
+      <c r="K66" s="10" t="n">
+        <f aca="false">IF(J66&lt;1000,CEILING(J66,10)-1,CEILING(J66,50)-1)</f>
+        <v>719</v>
+      </c>
+      <c r="L66" s="9" t="n">
+        <f aca="false">K66-F66</f>
+        <v>282.77</v>
+      </c>
+      <c r="M66" s="11" t="n">
+        <f aca="false">IF(K66=0,"",L66/K66)</f>
+        <v>0.393282336578581</v>
+      </c>
+      <c r="N66" s="11" t="n">
+        <f aca="false">IF(F66=0,"",K66/F66-1)</f>
+        <v>0.648213098594778</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F67" s="5" t="n">
+        <v>509.54</v>
+      </c>
+      <c r="G67" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F67,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H67" s="7"/>
+      <c r="I67" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F67,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J67" s="9" t="n">
+        <f aca="false">IF(H67="",MAX(F67*(1+G67),I67),F67*(1+H67))</f>
+        <v>840.741</v>
+      </c>
+      <c r="K67" s="10" t="n">
+        <f aca="false">IF(J67&lt;1000,CEILING(J67,10)-1,CEILING(J67,50)-1)</f>
+        <v>849</v>
+      </c>
+      <c r="L67" s="9" t="n">
+        <f aca="false">K67-F67</f>
+        <v>339.46</v>
+      </c>
+      <c r="M67" s="11" t="n">
+        <f aca="false">IF(K67=0,"",L67/K67)</f>
+        <v>0.399835100117786</v>
+      </c>
+      <c r="N67" s="11" t="n">
+        <f aca="false">IF(F67=0,"",K67/F67-1)</f>
+        <v>0.66620873729246</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F68" s="5" t="n">
+        <v>145.06</v>
+      </c>
+      <c r="G68" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F68,Reglas!$A$5:$A$8,1))</f>
+        <v>0.8</v>
+      </c>
+      <c r="H68" s="7"/>
+      <c r="I68" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F68,Reglas!$A$5:$A$8,1))</f>
+        <v>0</v>
+      </c>
+      <c r="J68" s="9" t="n">
+        <f aca="false">IF(H68="",MAX(F68*(1+G68),I68),F68*(1+H68))</f>
+        <v>261.108</v>
+      </c>
+      <c r="K68" s="10" t="n">
+        <f aca="false">IF(J68&lt;1000,CEILING(J68,10)-1,CEILING(J68,50)-1)</f>
+        <v>269</v>
+      </c>
+      <c r="L68" s="9" t="n">
+        <f aca="false">K68-F68</f>
+        <v>123.94</v>
+      </c>
+      <c r="M68" s="11" t="n">
+        <f aca="false">IF(K68=0,"",L68/K68)</f>
+        <v>0.460743494423792</v>
+      </c>
+      <c r="N68" s="11" t="n">
+        <f aca="false">IF(F68=0,"",K68/F68-1)</f>
+        <v>0.854405073762581</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F69" s="5" t="n">
+        <v>157.44</v>
+      </c>
+      <c r="G69" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F69,Reglas!$A$5:$A$8,1))</f>
+        <v>0.8</v>
+      </c>
+      <c r="H69" s="7"/>
+      <c r="I69" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F69,Reglas!$A$5:$A$8,1))</f>
+        <v>0</v>
+      </c>
+      <c r="J69" s="9" t="n">
+        <f aca="false">IF(H69="",MAX(F69*(1+G69),I69),F69*(1+H69))</f>
+        <v>283.392</v>
+      </c>
+      <c r="K69" s="10" t="n">
+        <f aca="false">IF(J69&lt;1000,CEILING(J69,10)-1,CEILING(J69,50)-1)</f>
+        <v>289</v>
+      </c>
+      <c r="L69" s="9" t="n">
+        <f aca="false">K69-F69</f>
+        <v>131.56</v>
+      </c>
+      <c r="M69" s="11" t="n">
+        <f aca="false">IF(K69=0,"",L69/K69)</f>
+        <v>0.45522491349481</v>
+      </c>
+      <c r="N69" s="11" t="n">
+        <f aca="false">IF(F69=0,"",K69/F69-1)</f>
+        <v>0.835619918699187</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F70" s="5" t="n">
+        <v>327.59</v>
+      </c>
+      <c r="G70" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F70,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H70" s="7"/>
+      <c r="I70" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F70,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J70" s="9" t="n">
+        <f aca="false">IF(H70="",MAX(F70*(1+G70),I70),F70*(1+H70))</f>
+        <v>540.5235</v>
+      </c>
+      <c r="K70" s="10" t="n">
+        <f aca="false">IF(J70&lt;1000,CEILING(J70,10)-1,CEILING(J70,50)-1)</f>
+        <v>549</v>
+      </c>
+      <c r="L70" s="9" t="n">
+        <f aca="false">K70-F70</f>
+        <v>221.41</v>
+      </c>
+      <c r="M70" s="11" t="n">
+        <f aca="false">IF(K70=0,"",L70/K70)</f>
+        <v>0.403296903460838</v>
+      </c>
+      <c r="N70" s="11" t="n">
+        <f aca="false">IF(F70=0,"",K70/F70-1)</f>
+        <v>0.675875331969841</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="F71" s="5" t="n">
+        <v>416.39</v>
+      </c>
+      <c r="G71" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F71,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H71" s="7"/>
+      <c r="I71" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F71,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J71" s="9" t="n">
+        <f aca="false">IF(H71="",MAX(F71*(1+G71),I71),F71*(1+H71))</f>
+        <v>687.0435</v>
+      </c>
+      <c r="K71" s="10" t="n">
+        <f aca="false">IF(J71&lt;1000,CEILING(J71,10)-1,CEILING(J71,50)-1)</f>
+        <v>689</v>
+      </c>
+      <c r="L71" s="9" t="n">
+        <f aca="false">K71-F71</f>
+        <v>272.61</v>
+      </c>
+      <c r="M71" s="11" t="n">
+        <f aca="false">IF(K71=0,"",L71/K71)</f>
+        <v>0.395660377358491</v>
+      </c>
+      <c r="N71" s="11" t="n">
+        <f aca="false">IF(F71=0,"",K71/F71-1)</f>
+        <v>0.654698719950047</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F72" s="5" t="n">
+        <v>496.84</v>
+      </c>
+      <c r="G72" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F72,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H72" s="7"/>
+      <c r="I72" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F72,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J72" s="9" t="n">
+        <f aca="false">IF(H72="",MAX(F72*(1+G72),I72),F72*(1+H72))</f>
+        <v>819.786</v>
+      </c>
+      <c r="K72" s="10" t="n">
+        <f aca="false">IF(J72&lt;1000,CEILING(J72,10)-1,CEILING(J72,50)-1)</f>
+        <v>819</v>
+      </c>
+      <c r="L72" s="9" t="n">
+        <f aca="false">K72-F72</f>
+        <v>322.16</v>
+      </c>
+      <c r="M72" s="11" t="n">
+        <f aca="false">IF(K72=0,"",L72/K72)</f>
+        <v>0.393357753357753</v>
+      </c>
+      <c r="N72" s="11" t="n">
+        <f aca="false">IF(F72=0,"",K72/F72-1)</f>
+        <v>0.648418001771194</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F73" s="5" t="n">
+        <v>1405.86</v>
+      </c>
+      <c r="G73" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F73,Reglas!$A$5:$A$8,1))</f>
+        <v>0.45</v>
+      </c>
+      <c r="H73" s="7"/>
+      <c r="I73" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F73,Reglas!$A$5:$A$8,1))</f>
+        <v>1860</v>
+      </c>
+      <c r="J73" s="9" t="n">
+        <f aca="false">IF(H73="",MAX(F73*(1+G73),I73),F73*(1+H73))</f>
+        <v>2038.497</v>
+      </c>
+      <c r="K73" s="10" t="n">
+        <f aca="false">IF(J73&lt;1000,CEILING(J73,10)-1,CEILING(J73,50)-1)</f>
+        <v>2049</v>
+      </c>
+      <c r="L73" s="9" t="n">
+        <f aca="false">K73-F73</f>
+        <v>643.14</v>
+      </c>
+      <c r="M73" s="11" t="n">
+        <f aca="false">IF(K73=0,"",L73/K73)</f>
+        <v>0.313879941434846</v>
+      </c>
+      <c r="N73" s="11" t="n">
+        <f aca="false">IF(F73=0,"",K73/F73-1)</f>
         <v>0.457470871921813</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="F44" s="14" t="n">
-        <f aca="false">SUM(F5:F43)</f>
-        <v>20784</v>
-      </c>
-      <c r="G44" s="12"/>
-      <c r="H44" s="12"/>
-      <c r="I44" s="12"/>
-      <c r="J44" s="12"/>
-      <c r="K44" s="15" t="n">
-        <f aca="false">SUM(K5:K43)</f>
-        <v>33331</v>
-      </c>
-      <c r="L44" s="14" t="n">
-        <f aca="false">SUM(L5:L43)</f>
-        <v>12547</v>
-      </c>
-      <c r="M44" s="16" t="n">
-        <f aca="false">IF(K44=0,"",L44/K44)</f>
-        <v>0.376436350544538</v>
-      </c>
-      <c r="N44" s="12"/>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="12"/>
+      <c r="B74" s="12"/>
+      <c r="C74" s="12"/>
+      <c r="D74" s="12"/>
+      <c r="E74" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="F74" s="14" t="n">
+        <f aca="false">SUM(F5:F73)</f>
+        <v>33875.59</v>
+      </c>
+      <c r="G74" s="12"/>
+      <c r="H74" s="12"/>
+      <c r="I74" s="12"/>
+      <c r="J74" s="12"/>
+      <c r="K74" s="15" t="n">
+        <f aca="false">SUM(K5:K73)</f>
+        <v>54711</v>
+      </c>
+      <c r="L74" s="14" t="n">
+        <f aca="false">SUM(L5:L73)</f>
+        <v>20835.41</v>
+      </c>
+      <c r="M74" s="16" t="n">
+        <f aca="false">IF(K74=0,"",L74/K74)</f>
+        <v>0.380826707609073</v>
+      </c>
+      <c r="N74" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N43"/>
+  <autoFilter ref="A4:N73"/>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
   </mergeCells>
@@ -3102,7 +4752,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3110,16 +4760,16 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>107</v>
+        <v>167</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>108</v>
+        <v>168</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>109</v>
+        <v>169</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>110</v>
+        <v>170</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>14</v>
@@ -3130,44 +4780,44 @@
         <v>16</v>
       </c>
       <c r="B4" s="17" t="n">
-        <f aca="false">COUNTIF(Precios!$B$5:$B$43,A4)</f>
-        <v>15</v>
+        <f aca="false">COUNTIF(Precios!$B$5:$B$73,A4)</f>
+        <v>45</v>
       </c>
       <c r="C4" s="18" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$43,A4,Precios!$F$5:$F$43)</f>
-        <v>6706.02</v>
+        <f aca="false">SUMIF(Precios!$B$5:$B$73,A4,Precios!$F$5:$F$73)</f>
+        <v>19797.61</v>
       </c>
       <c r="D4" s="19" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$43,A4,Precios!$K$5:$K$43)</f>
-        <v>11015</v>
+        <f aca="false">SUMIF(Precios!$B$5:$B$73,A4,Precios!$K$5:$K$73)</f>
+        <v>32395</v>
       </c>
       <c r="E4" s="18" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$43,A4,Precios!$L$5:$L$43)</f>
-        <v>4308.98</v>
+        <f aca="false">SUMIF(Precios!$B$5:$B$73,A4,Precios!$L$5:$L$73)</f>
+        <v>12597.39</v>
       </c>
       <c r="F4" s="20" t="n">
         <f aca="false">IF(D4=0,"",E4/D4)</f>
-        <v>0.391192010894235</v>
+        <v>0.388868343880228</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="B5" s="17" t="n">
-        <f aca="false">COUNTIF(Precios!$B$5:$B$43,A5)</f>
+        <f aca="false">COUNTIF(Precios!$B$5:$B$73,A5)</f>
         <v>24</v>
       </c>
       <c r="C5" s="18" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$43,A5,Precios!$F$5:$F$43)</f>
+        <f aca="false">SUMIF(Precios!$B$5:$B$73,A5,Precios!$F$5:$F$73)</f>
         <v>14077.98</v>
       </c>
       <c r="D5" s="19" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$43,A5,Precios!$K$5:$K$43)</f>
+        <f aca="false">SUMIF(Precios!$B$5:$B$73,A5,Precios!$K$5:$K$73)</f>
         <v>22316</v>
       </c>
       <c r="E5" s="18" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$43,A5,Precios!$L$5:$L$43)</f>
+        <f aca="false">SUMIF(Precios!$B$5:$B$73,A5,Precios!$L$5:$L$73)</f>
         <v>8238.02</v>
       </c>
       <c r="F5" s="20" t="n">
@@ -3177,27 +4827,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>111</v>
+        <v>171</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">SUM(B4:B5)</f>
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">SUM(C4:C5)</f>
-        <v>20784</v>
+        <v>33875.59</v>
       </c>
       <c r="D6" s="15" t="n">
         <f aca="false">SUM(D4:D5)</f>
-        <v>33331</v>
+        <v>54711</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">SUM(E4:E5)</f>
-        <v>12547</v>
+        <v>20835.41</v>
       </c>
       <c r="F6" s="16" t="n">
         <f aca="false">IF(D6=0,"",E6/D6)</f>
-        <v>0.376436350544538</v>
+        <v>0.380826707609073</v>
       </c>
     </row>
   </sheetData>
@@ -3227,23 +4877,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
-        <v>113</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>114</v>
+        <v>174</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>115</v>
+        <v>175</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>116</v>
+        <v>176</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>10</v>
@@ -3254,7 +4904,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>117</v>
+        <v>177</v>
       </c>
       <c r="C5" s="23" t="n">
         <v>0.8</v>
@@ -3268,7 +4918,7 @@
         <v>300</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>118</v>
+        <v>178</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>0.65</v>
@@ -3283,7 +4933,7 @@
         <v>700</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>119</v>
+        <v>179</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>0.55</v>
@@ -3298,7 +4948,7 @@
         <v>1200</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>0.45</v>
@@ -3310,37 +4960,37 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>121</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="s">
-        <v>122</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="24" t="s">
-        <v>123</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="24" t="s">
-        <v>124</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="24" t="s">
-        <v>125</v>
+        <v>185</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="24" t="s">
-        <v>126</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="24" t="s">
-        <v>127</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -3370,7 +5020,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3378,13 +5028,13 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>131</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3392,11 +5042,11 @@
         <v>16</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>132</v>
+        <v>192</v>
       </c>
       <c r="C4" s="25"/>
       <c r="D4" s="17" t="s">
-        <v>133</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3404,56 +5054,56 @@
         <v>16</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>134</v>
+        <v>194</v>
       </c>
       <c r="C5" s="25"/>
       <c r="D5" s="17" t="s">
-        <v>133</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>135</v>
+        <v>195</v>
       </c>
       <c r="C6" s="25"/>
       <c r="D6" s="17" t="s">
-        <v>133</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="C7" s="25" t="n">
         <v>239.56</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>137</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="C8" s="25" t="n">
         <v>556.04</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>137</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>138</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Catálogo: 10 productos más de CW & BW e imágenes partidas
- Sartenes, juegos, cacerola y baterías nuevas (79 productos en total).
- 'Cacerola' para los D.OV24LID y 'Olla' para el STW24LID, para no
  confundirlos.
- Las imágenes PNG se parten en partes de máximo 15 productos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FUhhJ2BRdUSntnn7uyZg21
</commit_message>
<xml_diff>
--- a/catalogo-cocina/salida/precios_internos_cocina.xlsx
+++ b/catalogo-cocina/salida/precios_internos_cocina.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Pendientes" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Precios!$A$4:$N$73</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Precios!$A$4:$N$83</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +31,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="F74" authorId="0">
+    <comment ref="F84" authorId="0">
       <text>
         <r>
           <rPr>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="221">
   <si>
     <t xml:space="preserve">Lista de precios interna (NO compartir con clientes)</t>
   </si>
@@ -128,6 +128,18 @@
     <t xml:space="preserve">Sartén Essential Titanium Gris 24 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP24 J LY SIMPLICITY GREY VIOLINE MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Simplicity Gris 24 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FP26 J LY EVERYDAY TITANIUM BLACK MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén Everyday Titanium Negra 26 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">SARTEN 28 CM RJ CHARACTER</t>
   </si>
   <si>
@@ -188,6 +200,12 @@
     <t xml:space="preserve">Crepera Hard Titanium Expert 25 cm</t>
   </si>
   <si>
+    <t xml:space="preserve">FP30 B JUNKO PE XL INTENSE BLACK COFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sartén XL Intense Negra 30 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">FP24 B SOFIA PE G6 DELIGHT IND BEIGE SAN</t>
   </si>
   <si>
@@ -266,6 +284,12 @@
     <t xml:space="preserve">Juego de 2 sartenes Resist Intense</t>
   </si>
   <si>
+    <t xml:space="preserve">SET 2FP 20/26 IND HARDTITAPRO BLACK MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 2 sartenes Hard Titanium Pro</t>
+  </si>
+  <si>
     <t xml:space="preserve">JGO 20/24/28 CM BG TRENDY TITANIUM</t>
   </si>
   <si>
@@ -278,6 +302,12 @@
     <t xml:space="preserve">Juego de 3 sartenes Daily Expert</t>
   </si>
   <si>
+    <t xml:space="preserve">JGO STN 20/24/28 CM DELIGHT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de 3 sartenes Delight Beige</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ollas y cazos</t>
   </si>
   <si>
@@ -308,7 +338,7 @@
     <t xml:space="preserve">D.OV24LID LENEXLOW COCINA LIMP DRESS BLU</t>
   </si>
   <si>
-    <t xml:space="preserve">Olla Azul 24 cm con tapa</t>
+    <t xml:space="preserve">Cacerola Azul 24 cm con tapa</t>
   </si>
   <si>
     <t xml:space="preserve">STW24LID B LENA HARD TITANIUM + BLACK MX</t>
@@ -317,6 +347,12 @@
     <t xml:space="preserve">Olla Hard Titanium+ Black 24 cm con tapa</t>
   </si>
   <si>
+    <t xml:space="preserve">D.OV24LID B LENA HARD TITANIUM+ BLACK MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cacerola Hard Titanium+ Black 24 cm con tapa</t>
+  </si>
+  <si>
     <t xml:space="preserve">OLLA 20 CM C/T TRENDY TITANIUM</t>
   </si>
   <si>
@@ -368,12 +404,36 @@
     <t xml:space="preserve">Batería Excite Azul 14 piezas</t>
   </si>
   <si>
+    <t xml:space="preserve">SET 7PCES SS DUETTO + TEF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batería Duetto+ 7 piezas</t>
+  </si>
+  <si>
     <t xml:space="preserve">BATERIA INOX 6 PCS INTUITION</t>
   </si>
   <si>
     <t xml:space="preserve">Batería Intuition 6 piezas</t>
   </si>
   <si>
+    <t xml:space="preserve">T PERFORMA PRO 14PC SET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batería Performa Pro 14 piezas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INGENIO ESSENTIAL PTFE 14PC SET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batería Ingenio Essential 14 piezas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET 12PCS XL FORCE TWINKLE MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batería XL Force 12 piezas</t>
+  </si>
+  <si>
     <t xml:space="preserve">BATERIA 12PZS NERA</t>
   </si>
   <si>
@@ -633,6 +693,12 @@
   </si>
   <si>
     <t xml:space="preserve">BATERIA 17 PZS NEGRA EASY CARE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FP30 J LY SIMPLY COOK RED BUG MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JGO 20/24/30 SIMPLY COOK RED</t>
   </si>
   <si>
     <t xml:space="preserve">QUICK CHEF+</t>
@@ -1222,7 +1288,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N74"/>
+  <dimension ref="A1:N84"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1519,7 +1585,7 @@
         <v>27</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>141.55</v>
+        <v>131.98</v>
       </c>
       <c r="G9" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F9,Reglas!$A$5:$A$8,1))</f>
@@ -1532,23 +1598,23 @@
       </c>
       <c r="J9" s="9" t="n">
         <f aca="false">IF(H9="",MAX(F9*(1+G9),I9),F9*(1+H9))</f>
-        <v>254.79</v>
+        <v>237.564</v>
       </c>
       <c r="K9" s="10" t="n">
         <f aca="false">IF(J9&lt;1000,CEILING(J9,10)-1,CEILING(J9,50)-1)</f>
-        <v>259</v>
+        <v>239</v>
       </c>
       <c r="L9" s="9" t="n">
         <f aca="false">K9-F9</f>
-        <v>117.45</v>
+        <v>107.02</v>
       </c>
       <c r="M9" s="11" t="n">
         <f aca="false">IF(K9=0,"",L9/K9)</f>
-        <v>0.453474903474903</v>
+        <v>0.447782426778243</v>
       </c>
       <c r="N9" s="11" t="n">
         <f aca="false">IF(F9=0,"",K9/F9-1)</f>
-        <v>0.829742140586365</v>
+        <v>0.810880436429762</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1568,7 +1634,7 @@
         <v>29</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>140.1</v>
+        <v>136.37</v>
       </c>
       <c r="G10" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F10,Reglas!$A$5:$A$8,1))</f>
@@ -1581,23 +1647,23 @@
       </c>
       <c r="J10" s="9" t="n">
         <f aca="false">IF(H10="",MAX(F10*(1+G10),I10),F10*(1+H10))</f>
-        <v>252.18</v>
+        <v>245.466</v>
       </c>
       <c r="K10" s="10" t="n">
         <f aca="false">IF(J10&lt;1000,CEILING(J10,10)-1,CEILING(J10,50)-1)</f>
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="L10" s="9" t="n">
         <f aca="false">K10-F10</f>
-        <v>118.9</v>
+        <v>112.63</v>
       </c>
       <c r="M10" s="11" t="n">
         <f aca="false">IF(K10=0,"",L10/K10)</f>
-        <v>0.459073359073359</v>
+        <v>0.452329317269076</v>
       </c>
       <c r="N10" s="11" t="n">
         <f aca="false">IF(F10=0,"",K10/F10-1)</f>
-        <v>0.848679514632406</v>
+        <v>0.825914790643103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1617,7 +1683,7 @@
         <v>31</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>146.67</v>
+        <v>141.55</v>
       </c>
       <c r="G11" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F11,Reglas!$A$5:$A$8,1))</f>
@@ -1630,23 +1696,23 @@
       </c>
       <c r="J11" s="9" t="n">
         <f aca="false">IF(H11="",MAX(F11*(1+G11),I11),F11*(1+H11))</f>
-        <v>264.006</v>
+        <v>254.79</v>
       </c>
       <c r="K11" s="10" t="n">
         <f aca="false">IF(J11&lt;1000,CEILING(J11,10)-1,CEILING(J11,50)-1)</f>
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="L11" s="9" t="n">
         <f aca="false">K11-F11</f>
-        <v>122.33</v>
+        <v>117.45</v>
       </c>
       <c r="M11" s="11" t="n">
         <f aca="false">IF(K11=0,"",L11/K11)</f>
-        <v>0.454758364312268</v>
+        <v>0.453474903474903</v>
       </c>
       <c r="N11" s="11" t="n">
         <f aca="false">IF(F11=0,"",K11/F11-1)</f>
-        <v>0.834049226153951</v>
+        <v>0.829742140586365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1666,7 +1732,7 @@
         <v>33</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>151.2</v>
+        <v>140.1</v>
       </c>
       <c r="G12" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F12,Reglas!$A$5:$A$8,1))</f>
@@ -1679,23 +1745,23 @@
       </c>
       <c r="J12" s="9" t="n">
         <f aca="false">IF(H12="",MAX(F12*(1+G12),I12),F12*(1+H12))</f>
-        <v>272.16</v>
+        <v>252.18</v>
       </c>
       <c r="K12" s="10" t="n">
         <f aca="false">IF(J12&lt;1000,CEILING(J12,10)-1,CEILING(J12,50)-1)</f>
-        <v>279</v>
+        <v>259</v>
       </c>
       <c r="L12" s="9" t="n">
         <f aca="false">K12-F12</f>
-        <v>127.8</v>
+        <v>118.9</v>
       </c>
       <c r="M12" s="11" t="n">
         <f aca="false">IF(K12=0,"",L12/K12)</f>
-        <v>0.458064516129032</v>
+        <v>0.459073359073359</v>
       </c>
       <c r="N12" s="11" t="n">
         <f aca="false">IF(F12=0,"",K12/F12-1)</f>
-        <v>0.845238095238095</v>
+        <v>0.848679514632406</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1715,7 +1781,7 @@
         <v>35</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>158.83</v>
+        <v>146.67</v>
       </c>
       <c r="G13" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F13,Reglas!$A$5:$A$8,1))</f>
@@ -1728,23 +1794,23 @@
       </c>
       <c r="J13" s="9" t="n">
         <f aca="false">IF(H13="",MAX(F13*(1+G13),I13),F13*(1+H13))</f>
-        <v>285.894</v>
+        <v>264.006</v>
       </c>
       <c r="K13" s="10" t="n">
         <f aca="false">IF(J13&lt;1000,CEILING(J13,10)-1,CEILING(J13,50)-1)</f>
-        <v>289</v>
+        <v>269</v>
       </c>
       <c r="L13" s="9" t="n">
         <f aca="false">K13-F13</f>
-        <v>130.17</v>
+        <v>122.33</v>
       </c>
       <c r="M13" s="11" t="n">
         <f aca="false">IF(K13=0,"",L13/K13)</f>
-        <v>0.450415224913495</v>
+        <v>0.454758364312268</v>
       </c>
       <c r="N13" s="11" t="n">
         <f aca="false">IF(F13=0,"",K13/F13-1)</f>
-        <v>0.819555499590757</v>
+        <v>0.834049226153951</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1764,7 +1830,7 @@
         <v>37</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>202.07</v>
+        <v>151.2</v>
       </c>
       <c r="G14" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F14,Reglas!$A$5:$A$8,1))</f>
@@ -1777,23 +1843,23 @@
       </c>
       <c r="J14" s="9" t="n">
         <f aca="false">IF(H14="",MAX(F14*(1+G14),I14),F14*(1+H14))</f>
-        <v>363.726</v>
+        <v>272.16</v>
       </c>
       <c r="K14" s="10" t="n">
         <f aca="false">IF(J14&lt;1000,CEILING(J14,10)-1,CEILING(J14,50)-1)</f>
-        <v>369</v>
+        <v>279</v>
       </c>
       <c r="L14" s="9" t="n">
         <f aca="false">K14-F14</f>
-        <v>166.93</v>
+        <v>127.8</v>
       </c>
       <c r="M14" s="11" t="n">
         <f aca="false">IF(K14=0,"",L14/K14)</f>
-        <v>0.452384823848239</v>
+        <v>0.458064516129032</v>
       </c>
       <c r="N14" s="11" t="n">
         <f aca="false">IF(F14=0,"",K14/F14-1)</f>
-        <v>0.826099866382937</v>
+        <v>0.845238095238095</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1813,7 +1879,7 @@
         <v>39</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>214.17</v>
+        <v>158.83</v>
       </c>
       <c r="G15" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F15,Reglas!$A$5:$A$8,1))</f>
@@ -1826,23 +1892,23 @@
       </c>
       <c r="J15" s="9" t="n">
         <f aca="false">IF(H15="",MAX(F15*(1+G15),I15),F15*(1+H15))</f>
-        <v>385.506</v>
+        <v>285.894</v>
       </c>
       <c r="K15" s="10" t="n">
         <f aca="false">IF(J15&lt;1000,CEILING(J15,10)-1,CEILING(J15,50)-1)</f>
-        <v>389</v>
+        <v>289</v>
       </c>
       <c r="L15" s="9" t="n">
         <f aca="false">K15-F15</f>
-        <v>174.83</v>
+        <v>130.17</v>
       </c>
       <c r="M15" s="11" t="n">
         <f aca="false">IF(K15=0,"",L15/K15)</f>
-        <v>0.449434447300771</v>
+        <v>0.450415224913495</v>
       </c>
       <c r="N15" s="11" t="n">
         <f aca="false">IF(F15=0,"",K15/F15-1)</f>
-        <v>0.816314142970538</v>
+        <v>0.819555499590757</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1862,7 +1928,7 @@
         <v>41</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>216.46</v>
+        <v>202.07</v>
       </c>
       <c r="G16" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F16,Reglas!$A$5:$A$8,1))</f>
@@ -1875,23 +1941,23 @@
       </c>
       <c r="J16" s="9" t="n">
         <f aca="false">IF(H16="",MAX(F16*(1+G16),I16),F16*(1+H16))</f>
-        <v>389.628</v>
+        <v>363.726</v>
       </c>
       <c r="K16" s="10" t="n">
         <f aca="false">IF(J16&lt;1000,CEILING(J16,10)-1,CEILING(J16,50)-1)</f>
-        <v>389</v>
+        <v>369</v>
       </c>
       <c r="L16" s="9" t="n">
         <f aca="false">K16-F16</f>
-        <v>172.54</v>
+        <v>166.93</v>
       </c>
       <c r="M16" s="11" t="n">
         <f aca="false">IF(K16=0,"",L16/K16)</f>
-        <v>0.443547557840617</v>
+        <v>0.452384823848239</v>
       </c>
       <c r="N16" s="11" t="n">
         <f aca="false">IF(F16=0,"",K16/F16-1)</f>
-        <v>0.797098771135545</v>
+        <v>0.826099866382937</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1911,7 +1977,7 @@
         <v>43</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>226.69</v>
+        <v>214.17</v>
       </c>
       <c r="G17" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F17,Reglas!$A$5:$A$8,1))</f>
@@ -1924,23 +1990,23 @@
       </c>
       <c r="J17" s="9" t="n">
         <f aca="false">IF(H17="",MAX(F17*(1+G17),I17),F17*(1+H17))</f>
-        <v>408.042</v>
+        <v>385.506</v>
       </c>
       <c r="K17" s="10" t="n">
         <f aca="false">IF(J17&lt;1000,CEILING(J17,10)-1,CEILING(J17,50)-1)</f>
-        <v>409</v>
+        <v>389</v>
       </c>
       <c r="L17" s="9" t="n">
         <f aca="false">K17-F17</f>
-        <v>182.31</v>
+        <v>174.83</v>
       </c>
       <c r="M17" s="11" t="n">
         <f aca="false">IF(K17=0,"",L17/K17)</f>
-        <v>0.445745721271394</v>
+        <v>0.449434447300771</v>
       </c>
       <c r="N17" s="11" t="n">
         <f aca="false">IF(F17=0,"",K17/F17-1)</f>
-        <v>0.804226035555163</v>
+        <v>0.816314142970538</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1960,7 +2026,7 @@
         <v>45</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>229.98</v>
+        <v>216.46</v>
       </c>
       <c r="G18" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F18,Reglas!$A$5:$A$8,1))</f>
@@ -1973,23 +2039,23 @@
       </c>
       <c r="J18" s="9" t="n">
         <f aca="false">IF(H18="",MAX(F18*(1+G18),I18),F18*(1+H18))</f>
-        <v>413.964</v>
+        <v>389.628</v>
       </c>
       <c r="K18" s="10" t="n">
         <f aca="false">IF(J18&lt;1000,CEILING(J18,10)-1,CEILING(J18,50)-1)</f>
-        <v>419</v>
+        <v>389</v>
       </c>
       <c r="L18" s="9" t="n">
         <f aca="false">K18-F18</f>
-        <v>189.02</v>
+        <v>172.54</v>
       </c>
       <c r="M18" s="11" t="n">
         <f aca="false">IF(K18=0,"",L18/K18)</f>
-        <v>0.451121718377088</v>
+        <v>0.443547557840617</v>
       </c>
       <c r="N18" s="11" t="n">
         <f aca="false">IF(F18=0,"",K18/F18-1)</f>
-        <v>0.821897556309244</v>
+        <v>0.797098771135545</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2009,7 +2075,7 @@
         <v>47</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>254.22</v>
+        <v>226.69</v>
       </c>
       <c r="G19" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F19,Reglas!$A$5:$A$8,1))</f>
@@ -2022,23 +2088,23 @@
       </c>
       <c r="J19" s="9" t="n">
         <f aca="false">IF(H19="",MAX(F19*(1+G19),I19),F19*(1+H19))</f>
-        <v>457.596</v>
+        <v>408.042</v>
       </c>
       <c r="K19" s="10" t="n">
         <f aca="false">IF(J19&lt;1000,CEILING(J19,10)-1,CEILING(J19,50)-1)</f>
-        <v>459</v>
+        <v>409</v>
       </c>
       <c r="L19" s="9" t="n">
         <f aca="false">K19-F19</f>
-        <v>204.78</v>
+        <v>182.31</v>
       </c>
       <c r="M19" s="11" t="n">
         <f aca="false">IF(K19=0,"",L19/K19)</f>
-        <v>0.446143790849673</v>
+        <v>0.445745721271394</v>
       </c>
       <c r="N19" s="11" t="n">
         <f aca="false">IF(F19=0,"",K19/F19-1)</f>
-        <v>0.805522775548737</v>
+        <v>0.804226035555163</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2058,7 +2124,7 @@
         <v>49</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>294.26</v>
+        <v>229.98</v>
       </c>
       <c r="G20" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F20,Reglas!$A$5:$A$8,1))</f>
@@ -2071,23 +2137,23 @@
       </c>
       <c r="J20" s="9" t="n">
         <f aca="false">IF(H20="",MAX(F20*(1+G20),I20),F20*(1+H20))</f>
-        <v>529.668</v>
+        <v>413.964</v>
       </c>
       <c r="K20" s="10" t="n">
         <f aca="false">IF(J20&lt;1000,CEILING(J20,10)-1,CEILING(J20,50)-1)</f>
-        <v>529</v>
+        <v>419</v>
       </c>
       <c r="L20" s="9" t="n">
         <f aca="false">K20-F20</f>
-        <v>234.74</v>
+        <v>189.02</v>
       </c>
       <c r="M20" s="11" t="n">
         <f aca="false">IF(K20=0,"",L20/K20)</f>
-        <v>0.443742911153119</v>
+        <v>0.451121718377088</v>
       </c>
       <c r="N20" s="11" t="n">
         <f aca="false">IF(F20=0,"",K20/F20-1)</f>
-        <v>0.797729898729015</v>
+        <v>0.821897556309244</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2107,7 +2173,7 @@
         <v>51</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>292.49</v>
+        <v>237.59</v>
       </c>
       <c r="G21" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F21,Reglas!$A$5:$A$8,1))</f>
@@ -2120,23 +2186,23 @@
       </c>
       <c r="J21" s="9" t="n">
         <f aca="false">IF(H21="",MAX(F21*(1+G21),I21),F21*(1+H21))</f>
-        <v>526.482</v>
+        <v>427.662</v>
       </c>
       <c r="K21" s="10" t="n">
         <f aca="false">IF(J21&lt;1000,CEILING(J21,10)-1,CEILING(J21,50)-1)</f>
-        <v>529</v>
+        <v>429</v>
       </c>
       <c r="L21" s="9" t="n">
         <f aca="false">K21-F21</f>
-        <v>236.51</v>
+        <v>191.41</v>
       </c>
       <c r="M21" s="11" t="n">
         <f aca="false">IF(K21=0,"",L21/K21)</f>
-        <v>0.447088846880907</v>
+        <v>0.446177156177156</v>
       </c>
       <c r="N21" s="11" t="n">
         <f aca="false">IF(F21=0,"",K21/F21-1)</f>
-        <v>0.808608841327909</v>
+        <v>0.805631550149417</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2147,16 +2213,16 @@
         <v>16</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>54</v>
-      </c>
       <c r="F22" s="5" t="n">
-        <v>184</v>
+        <v>254.22</v>
       </c>
       <c r="G22" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F22,Reglas!$A$5:$A$8,1))</f>
@@ -2169,23 +2235,23 @@
       </c>
       <c r="J22" s="9" t="n">
         <f aca="false">IF(H22="",MAX(F22*(1+G22),I22),F22*(1+H22))</f>
-        <v>331.2</v>
+        <v>457.596</v>
       </c>
       <c r="K22" s="10" t="n">
         <f aca="false">IF(J22&lt;1000,CEILING(J22,10)-1,CEILING(J22,50)-1)</f>
-        <v>339</v>
+        <v>459</v>
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">K22-F22</f>
-        <v>155</v>
+        <v>204.78</v>
       </c>
       <c r="M22" s="11" t="n">
         <f aca="false">IF(K22=0,"",L22/K22)</f>
-        <v>0.457227138643068</v>
+        <v>0.446143790849673</v>
       </c>
       <c r="N22" s="11" t="n">
         <f aca="false">IF(F22=0,"",K22/F22-1)</f>
-        <v>0.842391304347826</v>
+        <v>0.805522775548737</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2196,16 +2262,16 @@
         <v>16</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="D23" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>56</v>
-      </c>
       <c r="F23" s="5" t="n">
-        <v>197.64</v>
+        <v>294.26</v>
       </c>
       <c r="G23" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F23,Reglas!$A$5:$A$8,1))</f>
@@ -2218,23 +2284,23 @@
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">IF(H23="",MAX(F23*(1+G23),I23),F23*(1+H23))</f>
-        <v>355.752</v>
+        <v>529.668</v>
       </c>
       <c r="K23" s="10" t="n">
         <f aca="false">IF(J23&lt;1000,CEILING(J23,10)-1,CEILING(J23,50)-1)</f>
-        <v>359</v>
+        <v>529</v>
       </c>
       <c r="L23" s="9" t="n">
         <f aca="false">K23-F23</f>
-        <v>161.36</v>
+        <v>234.74</v>
       </c>
       <c r="M23" s="11" t="n">
         <f aca="false">IF(K23=0,"",L23/K23)</f>
-        <v>0.449470752089137</v>
+        <v>0.443742911153119</v>
       </c>
       <c r="N23" s="11" t="n">
         <f aca="false">IF(F23=0,"",K23/F23-1)</f>
-        <v>0.816433920259057</v>
+        <v>0.797729898729015</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2245,16 +2311,16 @@
         <v>16</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="D24" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E24" s="4" t="s">
-        <v>54</v>
-      </c>
       <c r="F24" s="5" t="n">
-        <v>275.63</v>
+        <v>292.49</v>
       </c>
       <c r="G24" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F24,Reglas!$A$5:$A$8,1))</f>
@@ -2267,23 +2333,23 @@
       </c>
       <c r="J24" s="9" t="n">
         <f aca="false">IF(H24="",MAX(F24*(1+G24),I24),F24*(1+H24))</f>
-        <v>496.134</v>
+        <v>526.482</v>
       </c>
       <c r="K24" s="10" t="n">
         <f aca="false">IF(J24&lt;1000,CEILING(J24,10)-1,CEILING(J24,50)-1)</f>
-        <v>499</v>
+        <v>529</v>
       </c>
       <c r="L24" s="9" t="n">
         <f aca="false">K24-F24</f>
-        <v>223.37</v>
+        <v>236.51</v>
       </c>
       <c r="M24" s="11" t="n">
         <f aca="false">IF(K24=0,"",L24/K24)</f>
-        <v>0.447635270541082</v>
+        <v>0.447088846880907</v>
       </c>
       <c r="N24" s="11" t="n">
         <f aca="false">IF(F24=0,"",K24/F24-1)</f>
-        <v>0.810397997315242</v>
+        <v>0.808608841327909</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2294,45 +2360,45 @@
         <v>16</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>325.16</v>
+        <v>184</v>
       </c>
       <c r="G25" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F25,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H25" s="7"/>
       <c r="I25" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F25,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J25" s="9" t="n">
         <f aca="false">IF(H25="",MAX(F25*(1+G25),I25),F25*(1+H25))</f>
-        <v>540</v>
+        <v>331.2</v>
       </c>
       <c r="K25" s="10" t="n">
         <f aca="false">IF(J25&lt;1000,CEILING(J25,10)-1,CEILING(J25,50)-1)</f>
-        <v>539</v>
+        <v>339</v>
       </c>
       <c r="L25" s="9" t="n">
         <f aca="false">K25-F25</f>
-        <v>213.84</v>
+        <v>155</v>
       </c>
       <c r="M25" s="11" t="n">
         <f aca="false">IF(K25=0,"",L25/K25)</f>
-        <v>0.396734693877551</v>
+        <v>0.457227138643068</v>
       </c>
       <c r="N25" s="11" t="n">
         <f aca="false">IF(F25=0,"",K25/F25-1)</f>
-        <v>0.657645466847091</v>
+        <v>0.842391304347826</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2343,45 +2409,45 @@
         <v>16</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>359.45</v>
+        <v>197.64</v>
       </c>
       <c r="G26" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F26,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H26" s="7"/>
       <c r="I26" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F26,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J26" s="9" t="n">
         <f aca="false">IF(H26="",MAX(F26*(1+G26),I26),F26*(1+H26))</f>
-        <v>593.0925</v>
+        <v>355.752</v>
       </c>
       <c r="K26" s="10" t="n">
         <f aca="false">IF(J26&lt;1000,CEILING(J26,10)-1,CEILING(J26,50)-1)</f>
-        <v>599</v>
+        <v>359</v>
       </c>
       <c r="L26" s="9" t="n">
         <f aca="false">K26-F26</f>
-        <v>239.55</v>
+        <v>161.36</v>
       </c>
       <c r="M26" s="11" t="n">
         <f aca="false">IF(K26=0,"",L26/K26)</f>
-        <v>0.39991652754591</v>
+        <v>0.449470752089137</v>
       </c>
       <c r="N26" s="11" t="n">
         <f aca="false">IF(F26=0,"",K26/F26-1)</f>
-        <v>0.666434830991793</v>
+        <v>0.816433920259057</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2392,45 +2458,45 @@
         <v>16</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>362.45</v>
+        <v>275.63</v>
       </c>
       <c r="G27" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F27,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H27" s="7"/>
       <c r="I27" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F27,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J27" s="9" t="n">
         <f aca="false">IF(H27="",MAX(F27*(1+G27),I27),F27*(1+H27))</f>
-        <v>598.0425</v>
+        <v>496.134</v>
       </c>
       <c r="K27" s="10" t="n">
         <f aca="false">IF(J27&lt;1000,CEILING(J27,10)-1,CEILING(J27,50)-1)</f>
-        <v>599</v>
+        <v>499</v>
       </c>
       <c r="L27" s="9" t="n">
         <f aca="false">K27-F27</f>
-        <v>236.55</v>
+        <v>223.37</v>
       </c>
       <c r="M27" s="11" t="n">
         <f aca="false">IF(K27=0,"",L27/K27)</f>
-        <v>0.394908180300501</v>
+        <v>0.447635270541082</v>
       </c>
       <c r="N27" s="11" t="n">
         <f aca="false">IF(F27=0,"",K27/F27-1)</f>
-        <v>0.652641743688785</v>
+        <v>0.810397997315242</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2441,7 +2507,7 @@
         <v>16</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>64</v>
@@ -2450,7 +2516,7 @@
         <v>65</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>487.77</v>
+        <v>325.16</v>
       </c>
       <c r="G28" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F28,Reglas!$A$5:$A$8,1))</f>
@@ -2463,23 +2529,23 @@
       </c>
       <c r="J28" s="9" t="n">
         <f aca="false">IF(H28="",MAX(F28*(1+G28),I28),F28*(1+H28))</f>
-        <v>804.8205</v>
+        <v>540</v>
       </c>
       <c r="K28" s="10" t="n">
         <f aca="false">IF(J28&lt;1000,CEILING(J28,10)-1,CEILING(J28,50)-1)</f>
-        <v>809</v>
+        <v>539</v>
       </c>
       <c r="L28" s="9" t="n">
         <f aca="false">K28-F28</f>
-        <v>321.23</v>
+        <v>213.84</v>
       </c>
       <c r="M28" s="11" t="n">
         <f aca="false">IF(K28=0,"",L28/K28)</f>
-        <v>0.397070457354759</v>
+        <v>0.396734693877551</v>
       </c>
       <c r="N28" s="11" t="n">
         <f aca="false">IF(F28=0,"",K28/F28-1)</f>
-        <v>0.658568587654017</v>
+        <v>0.657645466847091</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2490,7 +2556,7 @@
         <v>16</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>66</v>
@@ -2499,7 +2565,7 @@
         <v>67</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>492.72</v>
+        <v>359.45</v>
       </c>
       <c r="G29" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F29,Reglas!$A$5:$A$8,1))</f>
@@ -2512,23 +2578,23 @@
       </c>
       <c r="J29" s="9" t="n">
         <f aca="false">IF(H29="",MAX(F29*(1+G29),I29),F29*(1+H29))</f>
-        <v>812.988</v>
+        <v>593.0925</v>
       </c>
       <c r="K29" s="10" t="n">
         <f aca="false">IF(J29&lt;1000,CEILING(J29,10)-1,CEILING(J29,50)-1)</f>
-        <v>819</v>
+        <v>599</v>
       </c>
       <c r="L29" s="9" t="n">
         <f aca="false">K29-F29</f>
-        <v>326.28</v>
+        <v>239.55</v>
       </c>
       <c r="M29" s="11" t="n">
         <f aca="false">IF(K29=0,"",L29/K29)</f>
-        <v>0.398388278388278</v>
+        <v>0.39991652754591</v>
       </c>
       <c r="N29" s="11" t="n">
         <f aca="false">IF(F29=0,"",K29/F29-1)</f>
-        <v>0.662201656113005</v>
+        <v>0.666434830991793</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2539,7 +2605,7 @@
         <v>16</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>68</v>
@@ -2548,7 +2614,7 @@
         <v>69</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>515.85</v>
+        <v>362.45</v>
       </c>
       <c r="G30" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F30,Reglas!$A$5:$A$8,1))</f>
@@ -2561,23 +2627,23 @@
       </c>
       <c r="J30" s="9" t="n">
         <f aca="false">IF(H30="",MAX(F30*(1+G30),I30),F30*(1+H30))</f>
-        <v>851.1525</v>
+        <v>598.0425</v>
       </c>
       <c r="K30" s="10" t="n">
         <f aca="false">IF(J30&lt;1000,CEILING(J30,10)-1,CEILING(J30,50)-1)</f>
-        <v>859</v>
+        <v>599</v>
       </c>
       <c r="L30" s="9" t="n">
         <f aca="false">K30-F30</f>
-        <v>343.15</v>
+        <v>236.55</v>
       </c>
       <c r="M30" s="11" t="n">
         <f aca="false">IF(K30=0,"",L30/K30)</f>
-        <v>0.399476135040745</v>
+        <v>0.394908180300501</v>
       </c>
       <c r="N30" s="11" t="n">
         <f aca="false">IF(F30=0,"",K30/F30-1)</f>
-        <v>0.665212755646021</v>
+        <v>0.652641743688785</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2588,7 +2654,7 @@
         <v>16</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>70</v>
@@ -2597,7 +2663,7 @@
         <v>71</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>558.88</v>
+        <v>487.77</v>
       </c>
       <c r="G31" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F31,Reglas!$A$5:$A$8,1))</f>
@@ -2610,23 +2676,23 @@
       </c>
       <c r="J31" s="9" t="n">
         <f aca="false">IF(H31="",MAX(F31*(1+G31),I31),F31*(1+H31))</f>
-        <v>922.152</v>
+        <v>804.8205</v>
       </c>
       <c r="K31" s="10" t="n">
         <f aca="false">IF(J31&lt;1000,CEILING(J31,10)-1,CEILING(J31,50)-1)</f>
-        <v>929</v>
+        <v>809</v>
       </c>
       <c r="L31" s="9" t="n">
         <f aca="false">K31-F31</f>
-        <v>370.12</v>
+        <v>321.23</v>
       </c>
       <c r="M31" s="11" t="n">
         <f aca="false">IF(K31=0,"",L31/K31)</f>
-        <v>0.398406889128095</v>
+        <v>0.397070457354759</v>
       </c>
       <c r="N31" s="11" t="n">
         <f aca="false">IF(F31=0,"",K31/F31-1)</f>
-        <v>0.662253077583739</v>
+        <v>0.658568587654017</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2637,7 +2703,7 @@
         <v>16</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>72</v>
@@ -2646,36 +2712,36 @@
         <v>73</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>705.08</v>
+        <v>492.72</v>
       </c>
       <c r="G32" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F32,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H32" s="7"/>
       <c r="I32" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F32,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J32" s="9" t="n">
         <f aca="false">IF(H32="",MAX(F32*(1+G32),I32),F32*(1+H32))</f>
-        <v>1155</v>
+        <v>812.988</v>
       </c>
       <c r="K32" s="10" t="n">
         <f aca="false">IF(J32&lt;1000,CEILING(J32,10)-1,CEILING(J32,50)-1)</f>
-        <v>1199</v>
+        <v>819</v>
       </c>
       <c r="L32" s="9" t="n">
         <f aca="false">K32-F32</f>
-        <v>493.92</v>
+        <v>326.28</v>
       </c>
       <c r="M32" s="11" t="n">
         <f aca="false">IF(K32=0,"",L32/K32)</f>
-        <v>0.411943286071726</v>
+        <v>0.398388278388278</v>
       </c>
       <c r="N32" s="11" t="n">
         <f aca="false">IF(F32=0,"",K32/F32-1)</f>
-        <v>0.700516253474783</v>
+        <v>0.662201656113005</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2686,7 +2752,7 @@
         <v>16</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>74</v>
@@ -2695,36 +2761,36 @@
         <v>75</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>821.52</v>
+        <v>515.85</v>
       </c>
       <c r="G33" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F33,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H33" s="7"/>
       <c r="I33" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F33,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J33" s="9" t="n">
         <f aca="false">IF(H33="",MAX(F33*(1+G33),I33),F33*(1+H33))</f>
-        <v>1273.356</v>
+        <v>851.1525</v>
       </c>
       <c r="K33" s="10" t="n">
         <f aca="false">IF(J33&lt;1000,CEILING(J33,10)-1,CEILING(J33,50)-1)</f>
-        <v>1299</v>
+        <v>859</v>
       </c>
       <c r="L33" s="9" t="n">
         <f aca="false">K33-F33</f>
-        <v>477.48</v>
+        <v>343.15</v>
       </c>
       <c r="M33" s="11" t="n">
         <f aca="false">IF(K33=0,"",L33/K33)</f>
-        <v>0.367575057736721</v>
+        <v>0.399476135040745</v>
       </c>
       <c r="N33" s="11" t="n">
         <f aca="false">IF(F33=0,"",K33/F33-1)</f>
-        <v>0.581215308209173</v>
+        <v>0.665212755646021</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2735,45 +2801,45 @@
         <v>16</v>
       </c>
       <c r="C34" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="E34" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E34" s="4" t="s">
-        <v>78</v>
-      </c>
       <c r="F34" s="5" t="n">
-        <v>150.28</v>
+        <v>558.88</v>
       </c>
       <c r="G34" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F34,Reglas!$A$5:$A$8,1))</f>
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="H34" s="7"/>
       <c r="I34" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F34,Reglas!$A$5:$A$8,1))</f>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="J34" s="9" t="n">
         <f aca="false">IF(H34="",MAX(F34*(1+G34),I34),F34*(1+H34))</f>
-        <v>270.504</v>
+        <v>922.152</v>
       </c>
       <c r="K34" s="10" t="n">
         <f aca="false">IF(J34&lt;1000,CEILING(J34,10)-1,CEILING(J34,50)-1)</f>
-        <v>279</v>
+        <v>929</v>
       </c>
       <c r="L34" s="9" t="n">
         <f aca="false">K34-F34</f>
-        <v>128.72</v>
+        <v>370.12</v>
       </c>
       <c r="M34" s="11" t="n">
         <f aca="false">IF(K34=0,"",L34/K34)</f>
-        <v>0.461362007168459</v>
+        <v>0.398406889128095</v>
       </c>
       <c r="N34" s="11" t="n">
         <f aca="false">IF(F34=0,"",K34/F34-1)</f>
-        <v>0.856534468991216</v>
+        <v>0.662253077583739</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2784,45 +2850,45 @@
         <v>16</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="D35" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E35" s="4" t="s">
-        <v>80</v>
-      </c>
       <c r="F35" s="5" t="n">
-        <v>174.54</v>
+        <v>591.11</v>
       </c>
       <c r="G35" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F35,Reglas!$A$5:$A$8,1))</f>
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F35,Reglas!$A$5:$A$8,1))</f>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="J35" s="9" t="n">
         <f aca="false">IF(H35="",MAX(F35*(1+G35),I35),F35*(1+H35))</f>
-        <v>314.172</v>
+        <v>975.3315</v>
       </c>
       <c r="K35" s="10" t="n">
         <f aca="false">IF(J35&lt;1000,CEILING(J35,10)-1,CEILING(J35,50)-1)</f>
-        <v>319</v>
+        <v>979</v>
       </c>
       <c r="L35" s="9" t="n">
         <f aca="false">K35-F35</f>
-        <v>144.46</v>
+        <v>387.89</v>
       </c>
       <c r="M35" s="11" t="n">
         <f aca="false">IF(K35=0,"",L35/K35)</f>
-        <v>0.452852664576803</v>
+        <v>0.396210418794688</v>
       </c>
       <c r="N35" s="11" t="n">
         <f aca="false">IF(F35=0,"",K35/F35-1)</f>
-        <v>0.827661281081701</v>
+        <v>0.656206120688197</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2833,45 +2899,45 @@
         <v>16</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="D36" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E36" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E36" s="4" t="s">
-        <v>82</v>
-      </c>
       <c r="F36" s="5" t="n">
-        <v>319.2</v>
+        <v>705.08</v>
       </c>
       <c r="G36" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F36,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H36" s="7"/>
       <c r="I36" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F36,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J36" s="9" t="n">
         <f aca="false">IF(H36="",MAX(F36*(1+G36),I36),F36*(1+H36))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="K36" s="10" t="n">
         <f aca="false">IF(J36&lt;1000,CEILING(J36,10)-1,CEILING(J36,50)-1)</f>
-        <v>539</v>
+        <v>1199</v>
       </c>
       <c r="L36" s="9" t="n">
         <f aca="false">K36-F36</f>
-        <v>219.8</v>
+        <v>493.92</v>
       </c>
       <c r="M36" s="11" t="n">
         <f aca="false">IF(K36=0,"",L36/K36)</f>
-        <v>0.407792207792208</v>
+        <v>0.411943286071726</v>
       </c>
       <c r="N36" s="11" t="n">
         <f aca="false">IF(F36=0,"",K36/F36-1)</f>
-        <v>0.68859649122807</v>
+        <v>0.700516253474783</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2882,45 +2948,45 @@
         <v>16</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="D37" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E37" s="4" t="s">
-        <v>84</v>
-      </c>
       <c r="F37" s="5" t="n">
-        <v>324.7</v>
+        <v>821.52</v>
       </c>
       <c r="G37" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F37,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H37" s="7"/>
       <c r="I37" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F37,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J37" s="9" t="n">
         <f aca="false">IF(H37="",MAX(F37*(1+G37),I37),F37*(1+H37))</f>
-        <v>540</v>
+        <v>1273.356</v>
       </c>
       <c r="K37" s="10" t="n">
         <f aca="false">IF(J37&lt;1000,CEILING(J37,10)-1,CEILING(J37,50)-1)</f>
-        <v>539</v>
+        <v>1299</v>
       </c>
       <c r="L37" s="9" t="n">
         <f aca="false">K37-F37</f>
-        <v>214.3</v>
+        <v>477.48</v>
       </c>
       <c r="M37" s="11" t="n">
         <f aca="false">IF(K37=0,"",L37/K37)</f>
-        <v>0.397588126159555</v>
+        <v>0.367575057736721</v>
       </c>
       <c r="N37" s="11" t="n">
         <f aca="false">IF(F37=0,"",K37/F37-1)</f>
-        <v>0.659993840468125</v>
+        <v>0.581215308209173</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2931,45 +2997,45 @@
         <v>16</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="D38" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E38" s="4" t="s">
-        <v>86</v>
-      </c>
       <c r="F38" s="5" t="n">
-        <v>401.75</v>
+        <v>881.32</v>
       </c>
       <c r="G38" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F38,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H38" s="7"/>
       <c r="I38" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F38,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J38" s="9" t="n">
         <f aca="false">IF(H38="",MAX(F38*(1+G38),I38),F38*(1+H38))</f>
-        <v>662.8875</v>
+        <v>1366.046</v>
       </c>
       <c r="K38" s="10" t="n">
         <f aca="false">IF(J38&lt;1000,CEILING(J38,10)-1,CEILING(J38,50)-1)</f>
-        <v>669</v>
+        <v>1399</v>
       </c>
       <c r="L38" s="9" t="n">
         <f aca="false">K38-F38</f>
-        <v>267.25</v>
+        <v>517.68</v>
       </c>
       <c r="M38" s="11" t="n">
         <f aca="false">IF(K38=0,"",L38/K38)</f>
-        <v>0.399476831091181</v>
+        <v>0.370035739814153</v>
       </c>
       <c r="N38" s="11" t="n">
         <f aca="false">IF(F38=0,"",K38/F38-1)</f>
-        <v>0.665214685749844</v>
+        <v>0.587391639813008</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2980,7 +3046,7 @@
         <v>16</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>87</v>
@@ -2989,36 +3055,36 @@
         <v>88</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>422.36</v>
+        <v>150.28</v>
       </c>
       <c r="G39" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F39,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H39" s="7"/>
       <c r="I39" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F39,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J39" s="9" t="n">
         <f aca="false">IF(H39="",MAX(F39*(1+G39),I39),F39*(1+H39))</f>
-        <v>696.894</v>
+        <v>270.504</v>
       </c>
       <c r="K39" s="10" t="n">
         <f aca="false">IF(J39&lt;1000,CEILING(J39,10)-1,CEILING(J39,50)-1)</f>
-        <v>699</v>
+        <v>279</v>
       </c>
       <c r="L39" s="9" t="n">
         <f aca="false">K39-F39</f>
-        <v>276.64</v>
+        <v>128.72</v>
       </c>
       <c r="M39" s="11" t="n">
         <f aca="false">IF(K39=0,"",L39/K39)</f>
-        <v>0.395765379113019</v>
+        <v>0.461362007168459</v>
       </c>
       <c r="N39" s="11" t="n">
         <f aca="false">IF(F39=0,"",K39/F39-1)</f>
-        <v>0.654986267638981</v>
+        <v>0.856534468991216</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3029,7 +3095,7 @@
         <v>16</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>89</v>
@@ -3038,36 +3104,36 @@
         <v>90</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>427.15</v>
+        <v>174.54</v>
       </c>
       <c r="G40" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F40,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="H40" s="7"/>
       <c r="I40" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F40,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="J40" s="9" t="n">
         <f aca="false">IF(H40="",MAX(F40*(1+G40),I40),F40*(1+H40))</f>
-        <v>704.7975</v>
+        <v>314.172</v>
       </c>
       <c r="K40" s="10" t="n">
         <f aca="false">IF(J40&lt;1000,CEILING(J40,10)-1,CEILING(J40,50)-1)</f>
-        <v>709</v>
+        <v>319</v>
       </c>
       <c r="L40" s="9" t="n">
         <f aca="false">K40-F40</f>
-        <v>281.85</v>
+        <v>144.46</v>
       </c>
       <c r="M40" s="11" t="n">
         <f aca="false">IF(K40=0,"",L40/K40)</f>
-        <v>0.3975317348378</v>
+        <v>0.452852664576803</v>
       </c>
       <c r="N40" s="11" t="n">
         <f aca="false">IF(F40=0,"",K40/F40-1)</f>
-        <v>0.659838464239729</v>
+        <v>0.827661281081701</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3078,7 +3144,7 @@
         <v>16</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>91</v>
@@ -3087,7 +3153,7 @@
         <v>92</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>532.85</v>
+        <v>319.2</v>
       </c>
       <c r="G41" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F41,Reglas!$A$5:$A$8,1))</f>
@@ -3100,23 +3166,23 @@
       </c>
       <c r="J41" s="9" t="n">
         <f aca="false">IF(H41="",MAX(F41*(1+G41),I41),F41*(1+H41))</f>
-        <v>879.2025</v>
+        <v>540</v>
       </c>
       <c r="K41" s="10" t="n">
         <f aca="false">IF(J41&lt;1000,CEILING(J41,10)-1,CEILING(J41,50)-1)</f>
-        <v>879</v>
+        <v>539</v>
       </c>
       <c r="L41" s="9" t="n">
         <f aca="false">K41-F41</f>
-        <v>346.15</v>
+        <v>219.8</v>
       </c>
       <c r="M41" s="11" t="n">
         <f aca="false">IF(K41=0,"",L41/K41)</f>
-        <v>0.393799772468714</v>
+        <v>0.407792207792208</v>
       </c>
       <c r="N41" s="11" t="n">
         <f aca="false">IF(F41=0,"",K41/F41-1)</f>
-        <v>0.649619968096087</v>
+        <v>0.68859649122807</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3127,16 +3193,16 @@
         <v>16</v>
       </c>
       <c r="C42" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D42" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="E42" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E42" s="4" t="s">
-        <v>95</v>
-      </c>
       <c r="F42" s="5" t="n">
-        <v>377.88</v>
+        <v>324.7</v>
       </c>
       <c r="G42" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F42,Reglas!$A$5:$A$8,1))</f>
@@ -3149,23 +3215,23 @@
       </c>
       <c r="J42" s="9" t="n">
         <f aca="false">IF(H42="",MAX(F42*(1+G42),I42),F42*(1+H42))</f>
-        <v>623.502</v>
+        <v>540</v>
       </c>
       <c r="K42" s="10" t="n">
         <f aca="false">IF(J42&lt;1000,CEILING(J42,10)-1,CEILING(J42,50)-1)</f>
-        <v>629</v>
+        <v>539</v>
       </c>
       <c r="L42" s="9" t="n">
         <f aca="false">K42-F42</f>
-        <v>251.12</v>
+        <v>214.3</v>
       </c>
       <c r="M42" s="11" t="n">
         <f aca="false">IF(K42=0,"",L42/K42)</f>
-        <v>0.399236883942766</v>
+        <v>0.397588126159555</v>
       </c>
       <c r="N42" s="11" t="n">
         <f aca="false">IF(F42=0,"",K42/F42-1)</f>
-        <v>0.664549592463216</v>
+        <v>0.659993840468125</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3176,45 +3242,45 @@
         <v>16</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D43" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="E43" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="F43" s="5" t="n">
-        <v>737.5</v>
+        <v>401.75</v>
       </c>
       <c r="G43" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F43,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H43" s="7"/>
       <c r="I43" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F43,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J43" s="9" t="n">
         <f aca="false">IF(H43="",MAX(F43*(1+G43),I43),F43*(1+H43))</f>
-        <v>1155</v>
+        <v>662.8875</v>
       </c>
       <c r="K43" s="10" t="n">
         <f aca="false">IF(J43&lt;1000,CEILING(J43,10)-1,CEILING(J43,50)-1)</f>
-        <v>1199</v>
+        <v>669</v>
       </c>
       <c r="L43" s="9" t="n">
         <f aca="false">K43-F43</f>
-        <v>461.5</v>
+        <v>267.25</v>
       </c>
       <c r="M43" s="11" t="n">
         <f aca="false">IF(K43=0,"",L43/K43)</f>
-        <v>0.384904086738949</v>
+        <v>0.399476831091181</v>
       </c>
       <c r="N43" s="11" t="n">
         <f aca="false">IF(F43=0,"",K43/F43-1)</f>
-        <v>0.625762711864407</v>
+        <v>0.665214685749844</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3225,45 +3291,45 @@
         <v>16</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D44" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E44" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="F44" s="5" t="n">
-        <v>866.93</v>
+        <v>422.36</v>
       </c>
       <c r="G44" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F44,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H44" s="7"/>
       <c r="I44" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F44,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J44" s="9" t="n">
         <f aca="false">IF(H44="",MAX(F44*(1+G44),I44),F44*(1+H44))</f>
-        <v>1343.7415</v>
+        <v>696.894</v>
       </c>
       <c r="K44" s="10" t="n">
         <f aca="false">IF(J44&lt;1000,CEILING(J44,10)-1,CEILING(J44,50)-1)</f>
-        <v>1349</v>
+        <v>699</v>
       </c>
       <c r="L44" s="9" t="n">
         <f aca="false">K44-F44</f>
-        <v>482.07</v>
+        <v>276.64</v>
       </c>
       <c r="M44" s="11" t="n">
         <f aca="false">IF(K44=0,"",L44/K44)</f>
-        <v>0.357353595255745</v>
+        <v>0.395765379113019</v>
       </c>
       <c r="N44" s="11" t="n">
         <f aca="false">IF(F44=0,"",K44/F44-1)</f>
-        <v>0.556065656973458</v>
+        <v>0.654986267638981</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3274,45 +3340,45 @@
         <v>16</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D45" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E45" s="4" t="s">
-        <v>101</v>
-      </c>
       <c r="F45" s="5" t="n">
-        <v>901.39</v>
+        <v>424.95</v>
       </c>
       <c r="G45" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F45,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H45" s="7"/>
       <c r="I45" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F45,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J45" s="9" t="n">
         <f aca="false">IF(H45="",MAX(F45*(1+G45),I45),F45*(1+H45))</f>
-        <v>1397.1545</v>
+        <v>701.1675</v>
       </c>
       <c r="K45" s="10" t="n">
         <f aca="false">IF(J45&lt;1000,CEILING(J45,10)-1,CEILING(J45,50)-1)</f>
-        <v>1399</v>
+        <v>709</v>
       </c>
       <c r="L45" s="9" t="n">
         <f aca="false">K45-F45</f>
-        <v>497.61</v>
+        <v>284.05</v>
       </c>
       <c r="M45" s="11" t="n">
         <f aca="false">IF(K45=0,"",L45/K45)</f>
-        <v>0.355689778413152</v>
+        <v>0.400634696755994</v>
       </c>
       <c r="N45" s="11" t="n">
         <f aca="false">IF(F45=0,"",K45/F45-1)</f>
-        <v>0.552047393470085</v>
+        <v>0.668431580185904</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3323,45 +3389,45 @@
         <v>16</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D46" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E46" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E46" s="4" t="s">
-        <v>103</v>
-      </c>
       <c r="F46" s="5" t="n">
-        <v>1012.41</v>
+        <v>427.15</v>
       </c>
       <c r="G46" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F46,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H46" s="7"/>
       <c r="I46" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F46,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J46" s="9" t="n">
         <f aca="false">IF(H46="",MAX(F46*(1+G46),I46),F46*(1+H46))</f>
-        <v>1569.2355</v>
+        <v>704.7975</v>
       </c>
       <c r="K46" s="10" t="n">
         <f aca="false">IF(J46&lt;1000,CEILING(J46,10)-1,CEILING(J46,50)-1)</f>
-        <v>1599</v>
+        <v>709</v>
       </c>
       <c r="L46" s="9" t="n">
         <f aca="false">K46-F46</f>
-        <v>586.59</v>
+        <v>281.85</v>
       </c>
       <c r="M46" s="11" t="n">
         <f aca="false">IF(K46=0,"",L46/K46)</f>
-        <v>0.366848030018762</v>
+        <v>0.3975317348378</v>
       </c>
       <c r="N46" s="11" t="n">
         <f aca="false">IF(F46=0,"",K46/F46-1)</f>
-        <v>0.57939965033929</v>
+        <v>0.659838464239729</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3372,45 +3438,45 @@
         <v>16</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D47" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E47" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E47" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="F47" s="5" t="n">
-        <v>1047.3</v>
+        <v>532.85</v>
       </c>
       <c r="G47" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F47,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H47" s="7"/>
       <c r="I47" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F47,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J47" s="9" t="n">
         <f aca="false">IF(H47="",MAX(F47*(1+G47),I47),F47*(1+H47))</f>
-        <v>1623.315</v>
+        <v>879.2025</v>
       </c>
       <c r="K47" s="10" t="n">
         <f aca="false">IF(J47&lt;1000,CEILING(J47,10)-1,CEILING(J47,50)-1)</f>
-        <v>1649</v>
+        <v>879</v>
       </c>
       <c r="L47" s="9" t="n">
         <f aca="false">K47-F47</f>
-        <v>601.7</v>
+        <v>346.15</v>
       </c>
       <c r="M47" s="11" t="n">
         <f aca="false">IF(K47=0,"",L47/K47)</f>
-        <v>0.364887810794421</v>
+        <v>0.393799772468714</v>
       </c>
       <c r="N47" s="11" t="n">
         <f aca="false">IF(F47=0,"",K47/F47-1)</f>
-        <v>0.574524968967822</v>
+        <v>0.649619968096087</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3421,7 +3487,7 @@
         <v>16</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>106</v>
@@ -3430,36 +3496,36 @@
         <v>107</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>1275.69</v>
+        <v>377.88</v>
       </c>
       <c r="G48" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F48,Reglas!$A$5:$A$8,1))</f>
-        <v>0.45</v>
+        <v>0.65</v>
       </c>
       <c r="H48" s="7"/>
       <c r="I48" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F48,Reglas!$A$5:$A$8,1))</f>
-        <v>1860</v>
+        <v>540</v>
       </c>
       <c r="J48" s="9" t="n">
         <f aca="false">IF(H48="",MAX(F48*(1+G48),I48),F48*(1+H48))</f>
-        <v>1860</v>
+        <v>623.502</v>
       </c>
       <c r="K48" s="10" t="n">
         <f aca="false">IF(J48&lt;1000,CEILING(J48,10)-1,CEILING(J48,50)-1)</f>
-        <v>1899</v>
+        <v>629</v>
       </c>
       <c r="L48" s="9" t="n">
         <f aca="false">K48-F48</f>
-        <v>623.31</v>
+        <v>251.12</v>
       </c>
       <c r="M48" s="11" t="n">
         <f aca="false">IF(K48=0,"",L48/K48)</f>
-        <v>0.328230647709321</v>
+        <v>0.399236883942766</v>
       </c>
       <c r="N48" s="11" t="n">
         <f aca="false">IF(F48=0,"",K48/F48-1)</f>
-        <v>0.48860616607483</v>
+        <v>0.664549592463216</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3470,7 +3536,7 @@
         <v>16</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>108</v>
@@ -3479,36 +3545,36 @@
         <v>109</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>2411.07</v>
+        <v>737.5</v>
       </c>
       <c r="G49" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F49,Reglas!$A$5:$A$8,1))</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="H49" s="7"/>
       <c r="I49" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F49,Reglas!$A$5:$A$8,1))</f>
-        <v>1860</v>
+        <v>1155</v>
       </c>
       <c r="J49" s="9" t="n">
         <f aca="false">IF(H49="",MAX(F49*(1+G49),I49),F49*(1+H49))</f>
-        <v>3496.0515</v>
+        <v>1155</v>
       </c>
       <c r="K49" s="10" t="n">
         <f aca="false">IF(J49&lt;1000,CEILING(J49,10)-1,CEILING(J49,50)-1)</f>
-        <v>3499</v>
+        <v>1199</v>
       </c>
       <c r="L49" s="9" t="n">
         <f aca="false">K49-F49</f>
-        <v>1087.93</v>
+        <v>461.5</v>
       </c>
       <c r="M49" s="11" t="n">
         <f aca="false">IF(K49=0,"",L49/K49)</f>
-        <v>0.3109259788511</v>
+        <v>0.384904086738949</v>
       </c>
       <c r="N49" s="11" t="n">
         <f aca="false">IF(F49=0,"",K49/F49-1)</f>
-        <v>0.45122290103564</v>
+        <v>0.625762711864407</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3516,48 +3582,48 @@
         <v>46</v>
       </c>
       <c r="B50" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D50" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="E50" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D50" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>113</v>
-      </c>
       <c r="F50" s="5" t="n">
-        <v>362.5</v>
+        <v>866.93</v>
       </c>
       <c r="G50" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F50,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H50" s="7"/>
       <c r="I50" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F50,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J50" s="9" t="n">
         <f aca="false">IF(H50="",MAX(F50*(1+G50),I50),F50*(1+H50))</f>
-        <v>598.125</v>
+        <v>1343.7415</v>
       </c>
       <c r="K50" s="10" t="n">
         <f aca="false">IF(J50&lt;1000,CEILING(J50,10)-1,CEILING(J50,50)-1)</f>
-        <v>599</v>
+        <v>1349</v>
       </c>
       <c r="L50" s="9" t="n">
         <f aca="false">K50-F50</f>
-        <v>236.5</v>
+        <v>482.07</v>
       </c>
       <c r="M50" s="11" t="n">
         <f aca="false">IF(K50=0,"",L50/K50)</f>
-        <v>0.394824707846411</v>
+        <v>0.357353595255745</v>
       </c>
       <c r="N50" s="11" t="n">
         <f aca="false">IF(F50=0,"",K50/F50-1)</f>
-        <v>0.652413793103448</v>
+        <v>0.556065656973458</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3565,48 +3631,48 @@
         <v>47</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>384.06</v>
+        <v>901.39</v>
       </c>
       <c r="G51" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F51,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H51" s="7"/>
       <c r="I51" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F51,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J51" s="9" t="n">
         <f aca="false">IF(H51="",MAX(F51*(1+G51),I51),F51*(1+H51))</f>
-        <v>633.699</v>
+        <v>1397.1545</v>
       </c>
       <c r="K51" s="10" t="n">
         <f aca="false">IF(J51&lt;1000,CEILING(J51,10)-1,CEILING(J51,50)-1)</f>
-        <v>639</v>
+        <v>1399</v>
       </c>
       <c r="L51" s="9" t="n">
         <f aca="false">K51-F51</f>
-        <v>254.94</v>
+        <v>497.61</v>
       </c>
       <c r="M51" s="11" t="n">
         <f aca="false">IF(K51=0,"",L51/K51)</f>
-        <v>0.398967136150235</v>
+        <v>0.355689778413152</v>
       </c>
       <c r="N51" s="11" t="n">
         <f aca="false">IF(F51=0,"",K51/F51-1)</f>
-        <v>0.663802530854554</v>
+        <v>0.552047393470085</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3614,48 +3680,48 @@
         <v>48</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>384.59</v>
+        <v>1012.41</v>
       </c>
       <c r="G52" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F52,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H52" s="7"/>
       <c r="I52" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F52,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J52" s="9" t="n">
         <f aca="false">IF(H52="",MAX(F52*(1+G52),I52),F52*(1+H52))</f>
-        <v>634.5735</v>
+        <v>1569.2355</v>
       </c>
       <c r="K52" s="10" t="n">
         <f aca="false">IF(J52&lt;1000,CEILING(J52,10)-1,CEILING(J52,50)-1)</f>
-        <v>639</v>
+        <v>1599</v>
       </c>
       <c r="L52" s="9" t="n">
         <f aca="false">K52-F52</f>
-        <v>254.41</v>
+        <v>586.59</v>
       </c>
       <c r="M52" s="11" t="n">
         <f aca="false">IF(K52=0,"",L52/K52)</f>
-        <v>0.398137715179969</v>
+        <v>0.366848030018762</v>
       </c>
       <c r="N52" s="11" t="n">
         <f aca="false">IF(F52=0,"",K52/F52-1)</f>
-        <v>0.661509659637536</v>
+        <v>0.57939965033929</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3663,48 +3729,48 @@
         <v>49</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>419.93</v>
+        <v>1047.3</v>
       </c>
       <c r="G53" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F53,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H53" s="7"/>
       <c r="I53" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F53,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J53" s="9" t="n">
         <f aca="false">IF(H53="",MAX(F53*(1+G53),I53),F53*(1+H53))</f>
-        <v>692.8845</v>
+        <v>1623.315</v>
       </c>
       <c r="K53" s="10" t="n">
         <f aca="false">IF(J53&lt;1000,CEILING(J53,10)-1,CEILING(J53,50)-1)</f>
-        <v>699</v>
+        <v>1649</v>
       </c>
       <c r="L53" s="9" t="n">
         <f aca="false">K53-F53</f>
-        <v>279.07</v>
+        <v>601.7</v>
       </c>
       <c r="M53" s="11" t="n">
         <f aca="false">IF(K53=0,"",L53/K53)</f>
-        <v>0.399241773962804</v>
+        <v>0.364887810794421</v>
       </c>
       <c r="N53" s="11" t="n">
         <f aca="false">IF(F53=0,"",K53/F53-1)</f>
-        <v>0.66456314147596</v>
+        <v>0.574524968967822</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3712,48 +3778,48 @@
         <v>50</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>525.56</v>
+        <v>1104.95</v>
       </c>
       <c r="G54" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F54,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H54" s="7"/>
       <c r="I54" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F54,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J54" s="9" t="n">
         <f aca="false">IF(H54="",MAX(F54*(1+G54),I54),F54*(1+H54))</f>
-        <v>867.174</v>
+        <v>1712.6725</v>
       </c>
       <c r="K54" s="10" t="n">
         <f aca="false">IF(J54&lt;1000,CEILING(J54,10)-1,CEILING(J54,50)-1)</f>
-        <v>869</v>
+        <v>1749</v>
       </c>
       <c r="L54" s="9" t="n">
         <f aca="false">K54-F54</f>
-        <v>343.44</v>
+        <v>644.05</v>
       </c>
       <c r="M54" s="11" t="n">
         <f aca="false">IF(K54=0,"",L54/K54)</f>
-        <v>0.395212888377445</v>
+        <v>0.368238993710692</v>
       </c>
       <c r="N54" s="11" t="n">
         <f aca="false">IF(F54=0,"",K54/F54-1)</f>
-        <v>0.653474389222924</v>
+        <v>0.582877053260329</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3761,48 +3827,48 @@
         <v>51</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>550.83</v>
+        <v>1275.69</v>
       </c>
       <c r="G55" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F55,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H55" s="7"/>
       <c r="I55" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F55,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1860</v>
       </c>
       <c r="J55" s="9" t="n">
         <f aca="false">IF(H55="",MAX(F55*(1+G55),I55),F55*(1+H55))</f>
-        <v>908.8695</v>
+        <v>1860</v>
       </c>
       <c r="K55" s="10" t="n">
         <f aca="false">IF(J55&lt;1000,CEILING(J55,10)-1,CEILING(J55,50)-1)</f>
-        <v>909</v>
+        <v>1899</v>
       </c>
       <c r="L55" s="9" t="n">
         <f aca="false">K55-F55</f>
-        <v>358.17</v>
+        <v>623.31</v>
       </c>
       <c r="M55" s="11" t="n">
         <f aca="false">IF(K55=0,"",L55/K55)</f>
-        <v>0.394026402640264</v>
+        <v>0.328230647709321</v>
       </c>
       <c r="N55" s="11" t="n">
         <f aca="false">IF(F55=0,"",K55/F55-1)</f>
-        <v>0.650236915200697</v>
+        <v>0.48860616607483</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3810,48 +3876,48 @@
         <v>52</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>950.19</v>
+        <v>1381</v>
       </c>
       <c r="G56" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F56,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.45</v>
       </c>
       <c r="H56" s="7"/>
       <c r="I56" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F56,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>1860</v>
       </c>
       <c r="J56" s="9" t="n">
         <f aca="false">IF(H56="",MAX(F56*(1+G56),I56),F56*(1+H56))</f>
-        <v>1472.7945</v>
+        <v>2002.45</v>
       </c>
       <c r="K56" s="10" t="n">
         <f aca="false">IF(J56&lt;1000,CEILING(J56,10)-1,CEILING(J56,50)-1)</f>
-        <v>1499</v>
+        <v>2049</v>
       </c>
       <c r="L56" s="9" t="n">
         <f aca="false">K56-F56</f>
-        <v>548.81</v>
+        <v>668</v>
       </c>
       <c r="M56" s="11" t="n">
         <f aca="false">IF(K56=0,"",L56/K56)</f>
-        <v>0.366117411607739</v>
+        <v>0.326012689116642</v>
       </c>
       <c r="N56" s="11" t="n">
         <f aca="false">IF(F56=0,"",K56/F56-1)</f>
-        <v>0.577579220997906</v>
+        <v>0.483707458363505</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3859,48 +3925,48 @@
         <v>53</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C57" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D57" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D57" s="4" t="s">
-        <v>127</v>
-      </c>
       <c r="E57" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>978.67</v>
+        <v>1652.82</v>
       </c>
       <c r="G57" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F57,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.45</v>
       </c>
       <c r="H57" s="7"/>
       <c r="I57" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F57,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>1860</v>
       </c>
       <c r="J57" s="9" t="n">
         <f aca="false">IF(H57="",MAX(F57*(1+G57),I57),F57*(1+H57))</f>
-        <v>1516.9385</v>
+        <v>2396.589</v>
       </c>
       <c r="K57" s="10" t="n">
         <f aca="false">IF(J57&lt;1000,CEILING(J57,10)-1,CEILING(J57,50)-1)</f>
-        <v>1549</v>
+        <v>2399</v>
       </c>
       <c r="L57" s="9" t="n">
         <f aca="false">K57-F57</f>
-        <v>570.33</v>
+        <v>746.18</v>
       </c>
       <c r="M57" s="11" t="n">
         <f aca="false">IF(K57=0,"",L57/K57)</f>
-        <v>0.368192382182053</v>
+        <v>0.311037932471863</v>
       </c>
       <c r="N57" s="11" t="n">
         <f aca="false">IF(F57=0,"",K57/F57-1)</f>
-        <v>0.582760276702055</v>
+        <v>0.451458719037766</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3908,19 +3974,19 @@
         <v>54</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>1608.09</v>
+        <v>1869.42</v>
       </c>
       <c r="G58" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F58,Reglas!$A$5:$A$8,1))</f>
@@ -3933,23 +3999,23 @@
       </c>
       <c r="J58" s="9" t="n">
         <f aca="false">IF(H58="",MAX(F58*(1+G58),I58),F58*(1+H58))</f>
-        <v>2331.7305</v>
+        <v>2710.659</v>
       </c>
       <c r="K58" s="10" t="n">
         <f aca="false">IF(J58&lt;1000,CEILING(J58,10)-1,CEILING(J58,50)-1)</f>
-        <v>2349</v>
+        <v>2749</v>
       </c>
       <c r="L58" s="9" t="n">
         <f aca="false">K58-F58</f>
-        <v>740.91</v>
+        <v>879.58</v>
       </c>
       <c r="M58" s="11" t="n">
         <f aca="false">IF(K58=0,"",L58/K58)</f>
-        <v>0.315415070242656</v>
+        <v>0.319963623135686</v>
       </c>
       <c r="N58" s="11" t="n">
         <f aca="false">IF(F58=0,"",K58/F58-1)</f>
-        <v>0.460739137734828</v>
+        <v>0.470509569813097</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3957,19 +4023,19 @@
         <v>55</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>1645.59</v>
+        <v>2411.07</v>
       </c>
       <c r="G59" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F59,Reglas!$A$5:$A$8,1))</f>
@@ -3982,23 +4048,23 @@
       </c>
       <c r="J59" s="9" t="n">
         <f aca="false">IF(H59="",MAX(F59*(1+G59),I59),F59*(1+H59))</f>
-        <v>2386.1055</v>
+        <v>3496.0515</v>
       </c>
       <c r="K59" s="10" t="n">
         <f aca="false">IF(J59&lt;1000,CEILING(J59,10)-1,CEILING(J59,50)-1)</f>
-        <v>2399</v>
+        <v>3499</v>
       </c>
       <c r="L59" s="9" t="n">
         <f aca="false">K59-F59</f>
-        <v>753.41</v>
+        <v>1087.93</v>
       </c>
       <c r="M59" s="11" t="n">
         <f aca="false">IF(K59=0,"",L59/K59)</f>
-        <v>0.314051688203418</v>
+        <v>0.3109259788511</v>
       </c>
       <c r="N59" s="11" t="n">
         <f aca="false">IF(F59=0,"",K59/F59-1)</f>
-        <v>0.457835791418276</v>
+        <v>0.45122290103564</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4006,19 +4072,19 @@
         <v>56</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C60" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E60" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D60" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="E60" s="4" t="s">
-        <v>135</v>
-      </c>
       <c r="F60" s="5" t="n">
-        <v>321.42</v>
+        <v>362.5</v>
       </c>
       <c r="G60" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F60,Reglas!$A$5:$A$8,1))</f>
@@ -4031,23 +4097,23 @@
       </c>
       <c r="J60" s="9" t="n">
         <f aca="false">IF(H60="",MAX(F60*(1+G60),I60),F60*(1+H60))</f>
-        <v>540</v>
+        <v>598.125</v>
       </c>
       <c r="K60" s="10" t="n">
         <f aca="false">IF(J60&lt;1000,CEILING(J60,10)-1,CEILING(J60,50)-1)</f>
-        <v>539</v>
+        <v>599</v>
       </c>
       <c r="L60" s="9" t="n">
         <f aca="false">K60-F60</f>
-        <v>217.58</v>
+        <v>236.5</v>
       </c>
       <c r="M60" s="11" t="n">
         <f aca="false">IF(K60=0,"",L60/K60)</f>
-        <v>0.403673469387755</v>
+        <v>0.394824707846411</v>
       </c>
       <c r="N60" s="11" t="n">
         <f aca="false">IF(F60=0,"",K60/F60-1)</f>
-        <v>0.676933607118412</v>
+        <v>0.652413793103448</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4055,19 +4121,19 @@
         <v>57</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>321.42</v>
+        <v>384.06</v>
       </c>
       <c r="G61" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F61,Reglas!$A$5:$A$8,1))</f>
@@ -4080,23 +4146,23 @@
       </c>
       <c r="J61" s="9" t="n">
         <f aca="false">IF(H61="",MAX(F61*(1+G61),I61),F61*(1+H61))</f>
-        <v>540</v>
+        <v>633.699</v>
       </c>
       <c r="K61" s="10" t="n">
         <f aca="false">IF(J61&lt;1000,CEILING(J61,10)-1,CEILING(J61,50)-1)</f>
-        <v>539</v>
+        <v>639</v>
       </c>
       <c r="L61" s="9" t="n">
         <f aca="false">K61-F61</f>
-        <v>217.58</v>
+        <v>254.94</v>
       </c>
       <c r="M61" s="11" t="n">
         <f aca="false">IF(K61=0,"",L61/K61)</f>
-        <v>0.403673469387755</v>
+        <v>0.398967136150235</v>
       </c>
       <c r="N61" s="11" t="n">
         <f aca="false">IF(F61=0,"",K61/F61-1)</f>
-        <v>0.676933607118412</v>
+        <v>0.663802530854554</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4104,48 +4170,48 @@
         <v>58</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>823.36</v>
+        <v>384.59</v>
       </c>
       <c r="G62" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F62,Reglas!$A$5:$A$8,1))</f>
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="H62" s="7"/>
       <c r="I62" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F62,Reglas!$A$5:$A$8,1))</f>
-        <v>1155</v>
+        <v>540</v>
       </c>
       <c r="J62" s="9" t="n">
         <f aca="false">IF(H62="",MAX(F62*(1+G62),I62),F62*(1+H62))</f>
-        <v>1276.208</v>
+        <v>634.5735</v>
       </c>
       <c r="K62" s="10" t="n">
         <f aca="false">IF(J62&lt;1000,CEILING(J62,10)-1,CEILING(J62,50)-1)</f>
-        <v>1299</v>
+        <v>639</v>
       </c>
       <c r="L62" s="9" t="n">
         <f aca="false">K62-F62</f>
-        <v>475.64</v>
+        <v>254.41</v>
       </c>
       <c r="M62" s="11" t="n">
         <f aca="false">IF(K62=0,"",L62/K62)</f>
-        <v>0.366158583525789</v>
+        <v>0.398137715179969</v>
       </c>
       <c r="N62" s="11" t="n">
         <f aca="false">IF(F62=0,"",K62/F62-1)</f>
-        <v>0.577681694520016</v>
+        <v>0.661509659637536</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4153,48 +4219,48 @@
         <v>59</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>177.68</v>
+        <v>419.93</v>
       </c>
       <c r="G63" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F63,Reglas!$A$5:$A$8,1))</f>
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="H63" s="7"/>
       <c r="I63" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F63,Reglas!$A$5:$A$8,1))</f>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="J63" s="9" t="n">
         <f aca="false">IF(H63="",MAX(F63*(1+G63),I63),F63*(1+H63))</f>
-        <v>319.824</v>
+        <v>692.8845</v>
       </c>
       <c r="K63" s="10" t="n">
         <f aca="false">IF(J63&lt;1000,CEILING(J63,10)-1,CEILING(J63,50)-1)</f>
-        <v>319</v>
+        <v>699</v>
       </c>
       <c r="L63" s="9" t="n">
         <f aca="false">K63-F63</f>
-        <v>141.32</v>
+        <v>279.07</v>
       </c>
       <c r="M63" s="11" t="n">
         <f aca="false">IF(K63=0,"",L63/K63)</f>
-        <v>0.443009404388715</v>
+        <v>0.399241773962804</v>
       </c>
       <c r="N63" s="11" t="n">
         <f aca="false">IF(F63=0,"",K63/F63-1)</f>
-        <v>0.795362449347141</v>
+        <v>0.66456314147596</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4202,19 +4268,19 @@
         <v>60</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C64" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D64" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="D64" s="4" t="s">
-        <v>143</v>
-      </c>
       <c r="E64" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>305.32</v>
+        <v>525.56</v>
       </c>
       <c r="G64" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F64,Reglas!$A$5:$A$8,1))</f>
@@ -4227,23 +4293,23 @@
       </c>
       <c r="J64" s="9" t="n">
         <f aca="false">IF(H64="",MAX(F64*(1+G64),I64),F64*(1+H64))</f>
-        <v>540</v>
+        <v>867.174</v>
       </c>
       <c r="K64" s="10" t="n">
         <f aca="false">IF(J64&lt;1000,CEILING(J64,10)-1,CEILING(J64,50)-1)</f>
-        <v>539</v>
+        <v>869</v>
       </c>
       <c r="L64" s="9" t="n">
         <f aca="false">K64-F64</f>
-        <v>233.68</v>
+        <v>343.44</v>
       </c>
       <c r="M64" s="11" t="n">
         <f aca="false">IF(K64=0,"",L64/K64)</f>
-        <v>0.433543599257885</v>
+        <v>0.395212888377445</v>
       </c>
       <c r="N64" s="11" t="n">
         <f aca="false">IF(F64=0,"",K64/F64-1)</f>
-        <v>0.765360932791825</v>
+        <v>0.653474389222924</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4251,19 +4317,19 @@
         <v>61</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>423.82</v>
+        <v>550.83</v>
       </c>
       <c r="G65" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F65,Reglas!$A$5:$A$8,1))</f>
@@ -4276,23 +4342,23 @@
       </c>
       <c r="J65" s="9" t="n">
         <f aca="false">IF(H65="",MAX(F65*(1+G65),I65),F65*(1+H65))</f>
-        <v>699.303</v>
+        <v>908.8695</v>
       </c>
       <c r="K65" s="10" t="n">
         <f aca="false">IF(J65&lt;1000,CEILING(J65,10)-1,CEILING(J65,50)-1)</f>
-        <v>699</v>
+        <v>909</v>
       </c>
       <c r="L65" s="9" t="n">
         <f aca="false">K65-F65</f>
-        <v>275.18</v>
+        <v>358.17</v>
       </c>
       <c r="M65" s="11" t="n">
         <f aca="false">IF(K65=0,"",L65/K65)</f>
-        <v>0.393676680972818</v>
+        <v>0.394026402640264</v>
       </c>
       <c r="N65" s="11" t="n">
         <f aca="false">IF(F65=0,"",K65/F65-1)</f>
-        <v>0.649285073852107</v>
+        <v>0.650236915200697</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4300,48 +4366,48 @@
         <v>62</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>436.23</v>
+        <v>950.19</v>
       </c>
       <c r="G66" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F66,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H66" s="7"/>
       <c r="I66" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F66,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J66" s="9" t="n">
         <f aca="false">IF(H66="",MAX(F66*(1+G66),I66),F66*(1+H66))</f>
-        <v>719.7795</v>
+        <v>1472.7945</v>
       </c>
       <c r="K66" s="10" t="n">
         <f aca="false">IF(J66&lt;1000,CEILING(J66,10)-1,CEILING(J66,50)-1)</f>
-        <v>719</v>
+        <v>1499</v>
       </c>
       <c r="L66" s="9" t="n">
         <f aca="false">K66-F66</f>
-        <v>282.77</v>
+        <v>548.81</v>
       </c>
       <c r="M66" s="11" t="n">
         <f aca="false">IF(K66=0,"",L66/K66)</f>
-        <v>0.393282336578581</v>
+        <v>0.366117411607739</v>
       </c>
       <c r="N66" s="11" t="n">
         <f aca="false">IF(F66=0,"",K66/F66-1)</f>
-        <v>0.648213098594778</v>
+        <v>0.577579220997906</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4349,48 +4415,48 @@
         <v>63</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C67" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D67" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="D67" s="4" t="s">
-        <v>150</v>
-      </c>
       <c r="E67" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>509.54</v>
+        <v>978.67</v>
       </c>
       <c r="G67" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F67,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H67" s="7"/>
       <c r="I67" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F67,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J67" s="9" t="n">
         <f aca="false">IF(H67="",MAX(F67*(1+G67),I67),F67*(1+H67))</f>
-        <v>840.741</v>
+        <v>1516.9385</v>
       </c>
       <c r="K67" s="10" t="n">
         <f aca="false">IF(J67&lt;1000,CEILING(J67,10)-1,CEILING(J67,50)-1)</f>
-        <v>849</v>
+        <v>1549</v>
       </c>
       <c r="L67" s="9" t="n">
         <f aca="false">K67-F67</f>
-        <v>339.46</v>
+        <v>570.33</v>
       </c>
       <c r="M67" s="11" t="n">
         <f aca="false">IF(K67=0,"",L67/K67)</f>
-        <v>0.399835100117786</v>
+        <v>0.368192382182053</v>
       </c>
       <c r="N67" s="11" t="n">
         <f aca="false">IF(F67=0,"",K67/F67-1)</f>
-        <v>0.66620873729246</v>
+        <v>0.582760276702055</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4398,48 +4464,48 @@
         <v>64</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F68" s="5" t="n">
-        <v>145.06</v>
+        <v>1608.09</v>
       </c>
       <c r="G68" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F68,Reglas!$A$5:$A$8,1))</f>
-        <v>0.8</v>
+        <v>0.45</v>
       </c>
       <c r="H68" s="7"/>
       <c r="I68" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F68,Reglas!$A$5:$A$8,1))</f>
-        <v>0</v>
+        <v>1860</v>
       </c>
       <c r="J68" s="9" t="n">
         <f aca="false">IF(H68="",MAX(F68*(1+G68),I68),F68*(1+H68))</f>
-        <v>261.108</v>
+        <v>2331.7305</v>
       </c>
       <c r="K68" s="10" t="n">
         <f aca="false">IF(J68&lt;1000,CEILING(J68,10)-1,CEILING(J68,50)-1)</f>
-        <v>269</v>
+        <v>2349</v>
       </c>
       <c r="L68" s="9" t="n">
         <f aca="false">K68-F68</f>
-        <v>123.94</v>
+        <v>740.91</v>
       </c>
       <c r="M68" s="11" t="n">
         <f aca="false">IF(K68=0,"",L68/K68)</f>
-        <v>0.460743494423792</v>
+        <v>0.315415070242656</v>
       </c>
       <c r="N68" s="11" t="n">
         <f aca="false">IF(F68=0,"",K68/F68-1)</f>
-        <v>0.854405073762581</v>
+        <v>0.460739137734828</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4447,48 +4513,48 @@
         <v>65</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C69" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="E69" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D69" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E69" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="F69" s="5" t="n">
-        <v>157.44</v>
+        <v>1645.59</v>
       </c>
       <c r="G69" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F69,Reglas!$A$5:$A$8,1))</f>
-        <v>0.8</v>
+        <v>0.45</v>
       </c>
       <c r="H69" s="7"/>
       <c r="I69" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F69,Reglas!$A$5:$A$8,1))</f>
-        <v>0</v>
+        <v>1860</v>
       </c>
       <c r="J69" s="9" t="n">
         <f aca="false">IF(H69="",MAX(F69*(1+G69),I69),F69*(1+H69))</f>
-        <v>283.392</v>
+        <v>2386.1055</v>
       </c>
       <c r="K69" s="10" t="n">
         <f aca="false">IF(J69&lt;1000,CEILING(J69,10)-1,CEILING(J69,50)-1)</f>
-        <v>289</v>
+        <v>2399</v>
       </c>
       <c r="L69" s="9" t="n">
         <f aca="false">K69-F69</f>
-        <v>131.56</v>
+        <v>753.41</v>
       </c>
       <c r="M69" s="11" t="n">
         <f aca="false">IF(K69=0,"",L69/K69)</f>
-        <v>0.45522491349481</v>
+        <v>0.314051688203418</v>
       </c>
       <c r="N69" s="11" t="n">
         <f aca="false">IF(F69=0,"",K69/F69-1)</f>
-        <v>0.835619918699187</v>
+        <v>0.457835791418276</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4496,19 +4562,19 @@
         <v>66</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>327.59</v>
+        <v>321.42</v>
       </c>
       <c r="G70" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F70,Reglas!$A$5:$A$8,1))</f>
@@ -4521,23 +4587,23 @@
       </c>
       <c r="J70" s="9" t="n">
         <f aca="false">IF(H70="",MAX(F70*(1+G70),I70),F70*(1+H70))</f>
-        <v>540.5235</v>
+        <v>540</v>
       </c>
       <c r="K70" s="10" t="n">
         <f aca="false">IF(J70&lt;1000,CEILING(J70,10)-1,CEILING(J70,50)-1)</f>
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="L70" s="9" t="n">
         <f aca="false">K70-F70</f>
-        <v>221.41</v>
+        <v>217.58</v>
       </c>
       <c r="M70" s="11" t="n">
         <f aca="false">IF(K70=0,"",L70/K70)</f>
-        <v>0.403296903460838</v>
+        <v>0.403673469387755</v>
       </c>
       <c r="N70" s="11" t="n">
         <f aca="false">IF(F70=0,"",K70/F70-1)</f>
-        <v>0.675875331969841</v>
+        <v>0.676933607118412</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4545,19 +4611,19 @@
         <v>67</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F71" s="5" t="n">
-        <v>416.39</v>
+        <v>321.42</v>
       </c>
       <c r="G71" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F71,Reglas!$A$5:$A$8,1))</f>
@@ -4570,23 +4636,23 @@
       </c>
       <c r="J71" s="9" t="n">
         <f aca="false">IF(H71="",MAX(F71*(1+G71),I71),F71*(1+H71))</f>
-        <v>687.0435</v>
+        <v>540</v>
       </c>
       <c r="K71" s="10" t="n">
         <f aca="false">IF(J71&lt;1000,CEILING(J71,10)-1,CEILING(J71,50)-1)</f>
-        <v>689</v>
+        <v>539</v>
       </c>
       <c r="L71" s="9" t="n">
         <f aca="false">K71-F71</f>
-        <v>272.61</v>
+        <v>217.58</v>
       </c>
       <c r="M71" s="11" t="n">
         <f aca="false">IF(K71=0,"",L71/K71)</f>
-        <v>0.395660377358491</v>
+        <v>0.403673469387755</v>
       </c>
       <c r="N71" s="11" t="n">
         <f aca="false">IF(F71=0,"",K71/F71-1)</f>
-        <v>0.654698719950047</v>
+        <v>0.676933607118412</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4594,48 +4660,48 @@
         <v>68</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="F72" s="5" t="n">
-        <v>496.84</v>
+        <v>823.36</v>
       </c>
       <c r="G72" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F72,Reglas!$A$5:$A$8,1))</f>
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="H72" s="7"/>
       <c r="I72" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F72,Reglas!$A$5:$A$8,1))</f>
-        <v>540</v>
+        <v>1155</v>
       </c>
       <c r="J72" s="9" t="n">
         <f aca="false">IF(H72="",MAX(F72*(1+G72),I72),F72*(1+H72))</f>
-        <v>819.786</v>
+        <v>1276.208</v>
       </c>
       <c r="K72" s="10" t="n">
         <f aca="false">IF(J72&lt;1000,CEILING(J72,10)-1,CEILING(J72,50)-1)</f>
-        <v>819</v>
+        <v>1299</v>
       </c>
       <c r="L72" s="9" t="n">
         <f aca="false">K72-F72</f>
-        <v>322.16</v>
+        <v>475.64</v>
       </c>
       <c r="M72" s="11" t="n">
         <f aca="false">IF(K72=0,"",L72/K72)</f>
-        <v>0.393357753357753</v>
+        <v>0.366158583525789</v>
       </c>
       <c r="N72" s="11" t="n">
         <f aca="false">IF(F72=0,"",K72/F72-1)</f>
-        <v>0.648418001771194</v>
+        <v>0.577681694520016</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4643,82 +4709,572 @@
         <v>69</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F73" s="5" t="n">
-        <v>1405.86</v>
+        <v>177.68</v>
       </c>
       <c r="G73" s="6" t="n">
         <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F73,Reglas!$A$5:$A$8,1))</f>
-        <v>0.45</v>
+        <v>0.8</v>
       </c>
       <c r="H73" s="7"/>
       <c r="I73" s="8" t="n">
         <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F73,Reglas!$A$5:$A$8,1))</f>
-        <v>1860</v>
+        <v>0</v>
       </c>
       <c r="J73" s="9" t="n">
         <f aca="false">IF(H73="",MAX(F73*(1+G73),I73),F73*(1+H73))</f>
-        <v>2038.497</v>
+        <v>319.824</v>
       </c>
       <c r="K73" s="10" t="n">
         <f aca="false">IF(J73&lt;1000,CEILING(J73,10)-1,CEILING(J73,50)-1)</f>
-        <v>2049</v>
+        <v>319</v>
       </c>
       <c r="L73" s="9" t="n">
         <f aca="false">K73-F73</f>
-        <v>643.14</v>
+        <v>141.32</v>
       </c>
       <c r="M73" s="11" t="n">
         <f aca="false">IF(K73=0,"",L73/K73)</f>
-        <v>0.313879941434846</v>
+        <v>0.443009404388715</v>
       </c>
       <c r="N73" s="11" t="n">
         <f aca="false">IF(F73=0,"",K73/F73-1)</f>
+        <v>0.795362449347141</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F74" s="5" t="n">
+        <v>305.32</v>
+      </c>
+      <c r="G74" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F74,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H74" s="7"/>
+      <c r="I74" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F74,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J74" s="9" t="n">
+        <f aca="false">IF(H74="",MAX(F74*(1+G74),I74),F74*(1+H74))</f>
+        <v>540</v>
+      </c>
+      <c r="K74" s="10" t="n">
+        <f aca="false">IF(J74&lt;1000,CEILING(J74,10)-1,CEILING(J74,50)-1)</f>
+        <v>539</v>
+      </c>
+      <c r="L74" s="9" t="n">
+        <f aca="false">K74-F74</f>
+        <v>233.68</v>
+      </c>
+      <c r="M74" s="11" t="n">
+        <f aca="false">IF(K74=0,"",L74/K74)</f>
+        <v>0.433543599257885</v>
+      </c>
+      <c r="N74" s="11" t="n">
+        <f aca="false">IF(F74=0,"",K74/F74-1)</f>
+        <v>0.765360932791825</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F75" s="5" t="n">
+        <v>423.82</v>
+      </c>
+      <c r="G75" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F75,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H75" s="7"/>
+      <c r="I75" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F75,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J75" s="9" t="n">
+        <f aca="false">IF(H75="",MAX(F75*(1+G75),I75),F75*(1+H75))</f>
+        <v>699.303</v>
+      </c>
+      <c r="K75" s="10" t="n">
+        <f aca="false">IF(J75&lt;1000,CEILING(J75,10)-1,CEILING(J75,50)-1)</f>
+        <v>699</v>
+      </c>
+      <c r="L75" s="9" t="n">
+        <f aca="false">K75-F75</f>
+        <v>275.18</v>
+      </c>
+      <c r="M75" s="11" t="n">
+        <f aca="false">IF(K75=0,"",L75/K75)</f>
+        <v>0.393676680972818</v>
+      </c>
+      <c r="N75" s="11" t="n">
+        <f aca="false">IF(F75=0,"",K75/F75-1)</f>
+        <v>0.649285073852107</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="F76" s="5" t="n">
+        <v>436.23</v>
+      </c>
+      <c r="G76" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F76,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H76" s="7"/>
+      <c r="I76" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F76,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J76" s="9" t="n">
+        <f aca="false">IF(H76="",MAX(F76*(1+G76),I76),F76*(1+H76))</f>
+        <v>719.7795</v>
+      </c>
+      <c r="K76" s="10" t="n">
+        <f aca="false">IF(J76&lt;1000,CEILING(J76,10)-1,CEILING(J76,50)-1)</f>
+        <v>719</v>
+      </c>
+      <c r="L76" s="9" t="n">
+        <f aca="false">K76-F76</f>
+        <v>282.77</v>
+      </c>
+      <c r="M76" s="11" t="n">
+        <f aca="false">IF(K76=0,"",L76/K76)</f>
+        <v>0.393282336578581</v>
+      </c>
+      <c r="N76" s="11" t="n">
+        <f aca="false">IF(F76=0,"",K76/F76-1)</f>
+        <v>0.648213098594778</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F77" s="5" t="n">
+        <v>509.54</v>
+      </c>
+      <c r="G77" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F77,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H77" s="7"/>
+      <c r="I77" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F77,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J77" s="9" t="n">
+        <f aca="false">IF(H77="",MAX(F77*(1+G77),I77),F77*(1+H77))</f>
+        <v>840.741</v>
+      </c>
+      <c r="K77" s="10" t="n">
+        <f aca="false">IF(J77&lt;1000,CEILING(J77,10)-1,CEILING(J77,50)-1)</f>
+        <v>849</v>
+      </c>
+      <c r="L77" s="9" t="n">
+        <f aca="false">K77-F77</f>
+        <v>339.46</v>
+      </c>
+      <c r="M77" s="11" t="n">
+        <f aca="false">IF(K77=0,"",L77/K77)</f>
+        <v>0.399835100117786</v>
+      </c>
+      <c r="N77" s="11" t="n">
+        <f aca="false">IF(F77=0,"",K77/F77-1)</f>
+        <v>0.66620873729246</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F78" s="5" t="n">
+        <v>145.06</v>
+      </c>
+      <c r="G78" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F78,Reglas!$A$5:$A$8,1))</f>
+        <v>0.8</v>
+      </c>
+      <c r="H78" s="7"/>
+      <c r="I78" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F78,Reglas!$A$5:$A$8,1))</f>
+        <v>0</v>
+      </c>
+      <c r="J78" s="9" t="n">
+        <f aca="false">IF(H78="",MAX(F78*(1+G78),I78),F78*(1+H78))</f>
+        <v>261.108</v>
+      </c>
+      <c r="K78" s="10" t="n">
+        <f aca="false">IF(J78&lt;1000,CEILING(J78,10)-1,CEILING(J78,50)-1)</f>
+        <v>269</v>
+      </c>
+      <c r="L78" s="9" t="n">
+        <f aca="false">K78-F78</f>
+        <v>123.94</v>
+      </c>
+      <c r="M78" s="11" t="n">
+        <f aca="false">IF(K78=0,"",L78/K78)</f>
+        <v>0.460743494423792</v>
+      </c>
+      <c r="N78" s="11" t="n">
+        <f aca="false">IF(F78=0,"",K78/F78-1)</f>
+        <v>0.854405073762581</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="F79" s="5" t="n">
+        <v>157.44</v>
+      </c>
+      <c r="G79" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F79,Reglas!$A$5:$A$8,1))</f>
+        <v>0.8</v>
+      </c>
+      <c r="H79" s="7"/>
+      <c r="I79" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F79,Reglas!$A$5:$A$8,1))</f>
+        <v>0</v>
+      </c>
+      <c r="J79" s="9" t="n">
+        <f aca="false">IF(H79="",MAX(F79*(1+G79),I79),F79*(1+H79))</f>
+        <v>283.392</v>
+      </c>
+      <c r="K79" s="10" t="n">
+        <f aca="false">IF(J79&lt;1000,CEILING(J79,10)-1,CEILING(J79,50)-1)</f>
+        <v>289</v>
+      </c>
+      <c r="L79" s="9" t="n">
+        <f aca="false">K79-F79</f>
+        <v>131.56</v>
+      </c>
+      <c r="M79" s="11" t="n">
+        <f aca="false">IF(K79=0,"",L79/K79)</f>
+        <v>0.45522491349481</v>
+      </c>
+      <c r="N79" s="11" t="n">
+        <f aca="false">IF(F79=0,"",K79/F79-1)</f>
+        <v>0.835619918699187</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="F80" s="5" t="n">
+        <v>327.59</v>
+      </c>
+      <c r="G80" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F80,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H80" s="7"/>
+      <c r="I80" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F80,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J80" s="9" t="n">
+        <f aca="false">IF(H80="",MAX(F80*(1+G80),I80),F80*(1+H80))</f>
+        <v>540.5235</v>
+      </c>
+      <c r="K80" s="10" t="n">
+        <f aca="false">IF(J80&lt;1000,CEILING(J80,10)-1,CEILING(J80,50)-1)</f>
+        <v>549</v>
+      </c>
+      <c r="L80" s="9" t="n">
+        <f aca="false">K80-F80</f>
+        <v>221.41</v>
+      </c>
+      <c r="M80" s="11" t="n">
+        <f aca="false">IF(K80=0,"",L80/K80)</f>
+        <v>0.403296903460838</v>
+      </c>
+      <c r="N80" s="11" t="n">
+        <f aca="false">IF(F80=0,"",K80/F80-1)</f>
+        <v>0.675875331969841</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="F81" s="5" t="n">
+        <v>416.39</v>
+      </c>
+      <c r="G81" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F81,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H81" s="7"/>
+      <c r="I81" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F81,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J81" s="9" t="n">
+        <f aca="false">IF(H81="",MAX(F81*(1+G81),I81),F81*(1+H81))</f>
+        <v>687.0435</v>
+      </c>
+      <c r="K81" s="10" t="n">
+        <f aca="false">IF(J81&lt;1000,CEILING(J81,10)-1,CEILING(J81,50)-1)</f>
+        <v>689</v>
+      </c>
+      <c r="L81" s="9" t="n">
+        <f aca="false">K81-F81</f>
+        <v>272.61</v>
+      </c>
+      <c r="M81" s="11" t="n">
+        <f aca="false">IF(K81=0,"",L81/K81)</f>
+        <v>0.395660377358491</v>
+      </c>
+      <c r="N81" s="11" t="n">
+        <f aca="false">IF(F81=0,"",K81/F81-1)</f>
+        <v>0.654698719950047</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="F82" s="5" t="n">
+        <v>496.84</v>
+      </c>
+      <c r="G82" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F82,Reglas!$A$5:$A$8,1))</f>
+        <v>0.65</v>
+      </c>
+      <c r="H82" s="7"/>
+      <c r="I82" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F82,Reglas!$A$5:$A$8,1))</f>
+        <v>540</v>
+      </c>
+      <c r="J82" s="9" t="n">
+        <f aca="false">IF(H82="",MAX(F82*(1+G82),I82),F82*(1+H82))</f>
+        <v>819.786</v>
+      </c>
+      <c r="K82" s="10" t="n">
+        <f aca="false">IF(J82&lt;1000,CEILING(J82,10)-1,CEILING(J82,50)-1)</f>
+        <v>819</v>
+      </c>
+      <c r="L82" s="9" t="n">
+        <f aca="false">K82-F82</f>
+        <v>322.16</v>
+      </c>
+      <c r="M82" s="11" t="n">
+        <f aca="false">IF(K82=0,"",L82/K82)</f>
+        <v>0.393357753357753</v>
+      </c>
+      <c r="N82" s="11" t="n">
+        <f aca="false">IF(F82=0,"",K82/F82-1)</f>
+        <v>0.648418001771194</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="F83" s="5" t="n">
+        <v>1405.86</v>
+      </c>
+      <c r="G83" s="6" t="n">
+        <f aca="false">INDEX(Reglas!$C$5:$C$8,MATCH(F83,Reglas!$A$5:$A$8,1))</f>
+        <v>0.45</v>
+      </c>
+      <c r="H83" s="7"/>
+      <c r="I83" s="8" t="n">
+        <f aca="false">INDEX(Reglas!$D$5:$D$8,MATCH(F83,Reglas!$A$5:$A$8,1))</f>
+        <v>1860</v>
+      </c>
+      <c r="J83" s="9" t="n">
+        <f aca="false">IF(H83="",MAX(F83*(1+G83),I83),F83*(1+H83))</f>
+        <v>2038.497</v>
+      </c>
+      <c r="K83" s="10" t="n">
+        <f aca="false">IF(J83&lt;1000,CEILING(J83,10)-1,CEILING(J83,50)-1)</f>
+        <v>2049</v>
+      </c>
+      <c r="L83" s="9" t="n">
+        <f aca="false">K83-F83</f>
+        <v>643.14</v>
+      </c>
+      <c r="M83" s="11" t="n">
+        <f aca="false">IF(K83=0,"",L83/K83)</f>
+        <v>0.313879941434846</v>
+      </c>
+      <c r="N83" s="11" t="n">
+        <f aca="false">IF(F83=0,"",K83/F83-1)</f>
         <v>0.457470871921813</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="12"/>
-      <c r="B74" s="12"/>
-      <c r="C74" s="12"/>
-      <c r="D74" s="12"/>
-      <c r="E74" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="F74" s="14" t="n">
-        <f aca="false">SUM(F5:F73)</f>
-        <v>33875.59</v>
-      </c>
-      <c r="G74" s="12"/>
-      <c r="H74" s="12"/>
-      <c r="I74" s="12"/>
-      <c r="J74" s="12"/>
-      <c r="K74" s="15" t="n">
-        <f aca="false">SUM(K5:K73)</f>
-        <v>54711</v>
-      </c>
-      <c r="L74" s="14" t="n">
-        <f aca="false">SUM(L5:L73)</f>
-        <v>20835.41</v>
-      </c>
-      <c r="M74" s="16" t="n">
-        <f aca="false">IF(K74=0,"",L74/K74)</f>
-        <v>0.380826707609073</v>
-      </c>
-      <c r="N74" s="12"/>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="12"/>
+      <c r="B84" s="12"/>
+      <c r="C84" s="12"/>
+      <c r="D84" s="12"/>
+      <c r="E84" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="F84" s="14" t="n">
+        <f aca="false">SUM(F5:F83)</f>
+        <v>42287.1</v>
+      </c>
+      <c r="G84" s="12"/>
+      <c r="H84" s="12"/>
+      <c r="I84" s="12"/>
+      <c r="J84" s="12"/>
+      <c r="K84" s="15" t="n">
+        <f aca="false">SUM(K5:K83)</f>
+        <v>67661</v>
+      </c>
+      <c r="L84" s="14" t="n">
+        <f aca="false">SUM(L5:L83)</f>
+        <v>25373.9</v>
+      </c>
+      <c r="M84" s="16" t="n">
+        <f aca="false">IF(K84=0,"",L84/K84)</f>
+        <v>0.375015149051891</v>
+      </c>
+      <c r="N84" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N73"/>
+  <autoFilter ref="A4:N83"/>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
   </mergeCells>
@@ -4752,7 +5308,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>166</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4760,16 +5316,16 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>14</v>
@@ -4780,44 +5336,44 @@
         <v>16</v>
       </c>
       <c r="B4" s="17" t="n">
-        <f aca="false">COUNTIF(Precios!$B$5:$B$73,A4)</f>
-        <v>45</v>
+        <f aca="false">COUNTIF(Precios!$B$5:$B$83,A4)</f>
+        <v>55</v>
       </c>
       <c r="C4" s="18" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$73,A4,Precios!$F$5:$F$73)</f>
-        <v>19797.61</v>
+        <f aca="false">SUMIF(Precios!$B$5:$B$83,A4,Precios!$F$5:$F$83)</f>
+        <v>28209.12</v>
       </c>
       <c r="D4" s="19" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$73,A4,Precios!$K$5:$K$73)</f>
-        <v>32395</v>
+        <f aca="false">SUMIF(Precios!$B$5:$B$83,A4,Precios!$K$5:$K$83)</f>
+        <v>45345</v>
       </c>
       <c r="E4" s="18" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$73,A4,Precios!$L$5:$L$73)</f>
-        <v>12597.39</v>
+        <f aca="false">SUMIF(Precios!$B$5:$B$83,A4,Precios!$L$5:$L$83)</f>
+        <v>17135.88</v>
       </c>
       <c r="F4" s="20" t="n">
         <f aca="false">IF(D4=0,"",E4/D4)</f>
-        <v>0.388868343880228</v>
+        <v>0.377900099239166</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="B5" s="17" t="n">
-        <f aca="false">COUNTIF(Precios!$B$5:$B$73,A5)</f>
+        <f aca="false">COUNTIF(Precios!$B$5:$B$83,A5)</f>
         <v>24</v>
       </c>
       <c r="C5" s="18" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$73,A5,Precios!$F$5:$F$73)</f>
+        <f aca="false">SUMIF(Precios!$B$5:$B$83,A5,Precios!$F$5:$F$83)</f>
         <v>14077.98</v>
       </c>
       <c r="D5" s="19" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$73,A5,Precios!$K$5:$K$73)</f>
+        <f aca="false">SUMIF(Precios!$B$5:$B$83,A5,Precios!$K$5:$K$83)</f>
         <v>22316</v>
       </c>
       <c r="E5" s="18" t="n">
-        <f aca="false">SUMIF(Precios!$B$5:$B$73,A5,Precios!$L$5:$L$73)</f>
+        <f aca="false">SUMIF(Precios!$B$5:$B$83,A5,Precios!$L$5:$L$83)</f>
         <v>8238.02</v>
       </c>
       <c r="F5" s="20" t="n">
@@ -4827,27 +5383,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>171</v>
+        <v>191</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">SUM(B4:B5)</f>
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">SUM(C4:C5)</f>
-        <v>33875.59</v>
+        <v>42287.1</v>
       </c>
       <c r="D6" s="15" t="n">
         <f aca="false">SUM(D4:D5)</f>
-        <v>54711</v>
+        <v>67661</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">SUM(E4:E5)</f>
-        <v>20835.41</v>
+        <v>25373.9</v>
       </c>
       <c r="F6" s="16" t="n">
         <f aca="false">IF(D6=0,"",E6/D6)</f>
-        <v>0.380826707609073</v>
+        <v>0.375015149051891</v>
       </c>
     </row>
   </sheetData>
@@ -4877,23 +5433,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>172</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>10</v>
@@ -4904,7 +5460,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="C5" s="23" t="n">
         <v>0.8</v>
@@ -4918,7 +5474,7 @@
         <v>300</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>0.65</v>
@@ -4933,7 +5489,7 @@
         <v>700</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>179</v>
+        <v>199</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>0.55</v>
@@ -4948,7 +5504,7 @@
         <v>1200</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>0.45</v>
@@ -4960,37 +5516,37 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="24" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="24" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="24" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="24" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="24" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -5009,7 +5565,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -5020,7 +5576,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5028,13 +5584,13 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5042,11 +5598,11 @@
         <v>16</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="C4" s="25"/>
       <c r="D4" s="17" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5054,56 +5610,80 @@
         <v>16</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>194</v>
+        <v>214</v>
       </c>
       <c r="C5" s="25"/>
       <c r="D5" s="17" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>195</v>
+        <v>215</v>
       </c>
       <c r="C6" s="25"/>
       <c r="D6" s="17" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="C7" s="25" t="n">
-        <v>239.56</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="C7" s="25"/>
       <c r="D7" s="17" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="C8" s="25" t="n">
+        <v>217</v>
+      </c>
+      <c r="C8" s="25"/>
+      <c r="D8" s="17" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>239.56</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="C10" s="25" t="n">
         <v>556.04</v>
       </c>
-      <c r="D8" s="17" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>198</v>
+      <c r="D10" s="17" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>